<commit_message>
Estadisticos Segundo Parcial 20231 3NN
</commit_message>
<xml_diff>
--- a/Calificaciones20231.xlsx
+++ b/Calificaciones20231.xlsx
@@ -9820,7 +9820,7 @@
         <v>9</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I4">
         <v>9</v>
@@ -9856,7 +9856,7 @@
         <v>-1</v>
       </c>
       <c r="T4">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U4">
         <v>8</v>
@@ -9897,7 +9897,7 @@
         <v>8</v>
       </c>
       <c r="H5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I5">
         <v>9</v>
@@ -9933,7 +9933,7 @@
         <v>-1</v>
       </c>
       <c r="T5">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U5">
         <v>8</v>
@@ -9974,7 +9974,7 @@
         <v>10</v>
       </c>
       <c r="H6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I6">
         <v>9</v>
@@ -10010,7 +10010,7 @@
         <v>-1</v>
       </c>
       <c r="T6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U6">
         <v>8</v>
@@ -10051,7 +10051,7 @@
         <v>9</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I7">
         <v>9</v>
@@ -10128,7 +10128,7 @@
         <v>10</v>
       </c>
       <c r="H8">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I8">
         <v>9</v>
@@ -10205,7 +10205,7 @@
         <v>10</v>
       </c>
       <c r="H9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I9">
         <v>9</v>
@@ -10241,7 +10241,7 @@
         <v>-1</v>
       </c>
       <c r="T9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U9">
         <v>8</v>
@@ -10282,7 +10282,7 @@
         <v>5</v>
       </c>
       <c r="H10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I10">
         <v>9</v>
@@ -10359,7 +10359,7 @@
         <v>8</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I11">
         <v>9</v>
@@ -10436,7 +10436,7 @@
         <v>9</v>
       </c>
       <c r="H12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I12">
         <v>9</v>
@@ -10513,7 +10513,7 @@
         <v>8</v>
       </c>
       <c r="H13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I13">
         <v>9</v>
@@ -10549,7 +10549,7 @@
         <v>-1</v>
       </c>
       <c r="T13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U13">
         <v>8</v>
@@ -10590,7 +10590,7 @@
         <v>9</v>
       </c>
       <c r="H14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I14">
         <v>9</v>
@@ -10626,7 +10626,7 @@
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U14">
         <v>8</v>
@@ -10667,7 +10667,7 @@
         <v>8</v>
       </c>
       <c r="H15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I15">
         <v>9</v>
@@ -10744,7 +10744,7 @@
         <v>8</v>
       </c>
       <c r="H16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I16">
         <v>9</v>
@@ -10780,7 +10780,7 @@
         <v>-1</v>
       </c>
       <c r="T16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U16">
         <v>7</v>
@@ -10821,7 +10821,7 @@
         <v>8</v>
       </c>
       <c r="H17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I17">
         <v>9</v>
@@ -10898,7 +10898,7 @@
         <v>6</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I18">
         <v>9</v>
@@ -10975,7 +10975,7 @@
         <v>9</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I19">
         <v>9</v>
@@ -11052,7 +11052,7 @@
         <v>9</v>
       </c>
       <c r="H20">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I20">
         <v>9</v>
@@ -11088,7 +11088,7 @@
         <v>-1</v>
       </c>
       <c r="T20">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U20">
         <v>10</v>
@@ -11129,7 +11129,7 @@
         <v>5</v>
       </c>
       <c r="H21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I21">
         <v>9</v>
@@ -11206,7 +11206,7 @@
         <v>9</v>
       </c>
       <c r="H22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I22">
         <v>9</v>
@@ -11242,7 +11242,7 @@
         <v>-1</v>
       </c>
       <c r="T22">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U22">
         <v>8</v>
@@ -11283,7 +11283,7 @@
         <v>6</v>
       </c>
       <c r="H23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I23">
         <v>9</v>
@@ -11319,7 +11319,7 @@
         <v>-1</v>
       </c>
       <c r="T23">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U23">
         <v>7</v>
@@ -11360,7 +11360,7 @@
         <v>7</v>
       </c>
       <c r="H24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I24">
         <v>9</v>
@@ -11396,7 +11396,7 @@
         <v>-1</v>
       </c>
       <c r="T24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U24">
         <v>8</v>
@@ -11437,7 +11437,7 @@
         <v>8</v>
       </c>
       <c r="H25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I25">
         <v>9</v>
@@ -11514,7 +11514,7 @@
         <v>10</v>
       </c>
       <c r="H26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I26">
         <v>9</v>
@@ -11550,7 +11550,7 @@
         <v>-1</v>
       </c>
       <c r="T26">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U26">
         <v>8</v>
@@ -11591,7 +11591,7 @@
         <v>8</v>
       </c>
       <c r="H27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I27">
         <v>9</v>
@@ -11668,7 +11668,7 @@
         <v>9</v>
       </c>
       <c r="H28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I28">
         <v>9</v>
@@ -11745,7 +11745,7 @@
         <v>6</v>
       </c>
       <c r="H29">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I29">
         <v>9</v>
@@ -11822,7 +11822,7 @@
         <v>9</v>
       </c>
       <c r="H30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I30">
         <v>9</v>
@@ -11858,7 +11858,7 @@
         <v>-1</v>
       </c>
       <c r="T30">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U30">
         <v>8</v>
@@ -11899,7 +11899,7 @@
         <v>10</v>
       </c>
       <c r="H31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I31">
         <v>9</v>
@@ -11935,7 +11935,7 @@
         <v>-1</v>
       </c>
       <c r="T31">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U31">
         <v>8</v>
@@ -11976,7 +11976,7 @@
         <v>5</v>
       </c>
       <c r="H32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I32">
         <v>9</v>
@@ -12053,7 +12053,7 @@
         <v>10</v>
       </c>
       <c r="H33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I33">
         <v>9</v>
@@ -12130,7 +12130,7 @@
         <v>10</v>
       </c>
       <c r="H34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I34">
         <v>9</v>
@@ -12207,7 +12207,7 @@
         <v>9</v>
       </c>
       <c r="H35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I35">
         <v>9</v>
@@ -12243,7 +12243,7 @@
         <v>-1</v>
       </c>
       <c r="T35">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U35">
         <v>8</v>
@@ -14120,10 +14120,10 @@
         <v>6</v>
       </c>
       <c r="J26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="K26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L26">
         <v>10</v>
@@ -14159,7 +14159,7 @@
         <v>5</v>
       </c>
       <c r="W26">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X26">
         <v>10</v>
@@ -54662,7 +54662,7 @@
         <v>4</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I4">
         <v>6</v>
@@ -54698,7 +54698,7 @@
         <v>-1</v>
       </c>
       <c r="T4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U4">
         <v>7</v>
@@ -54739,7 +54739,7 @@
         <v>7</v>
       </c>
       <c r="H5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I5">
         <v>9</v>
@@ -54816,7 +54816,7 @@
         <v>6</v>
       </c>
       <c r="H6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I6">
         <v>7</v>
@@ -54893,7 +54893,7 @@
         <v>6</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I7">
         <v>6</v>
@@ -54970,7 +54970,7 @@
         <v>9</v>
       </c>
       <c r="H8">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I8">
         <v>9</v>
@@ -55047,7 +55047,7 @@
         <v>7</v>
       </c>
       <c r="H9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I9">
         <v>7</v>
@@ -55124,7 +55124,7 @@
         <v>4</v>
       </c>
       <c r="H10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I10">
         <v>5</v>
@@ -55201,7 +55201,7 @@
         <v>7</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I11">
         <v>7</v>
@@ -55278,7 +55278,7 @@
         <v>3</v>
       </c>
       <c r="H12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I12">
         <v>7</v>
@@ -55355,7 +55355,7 @@
         <v>9</v>
       </c>
       <c r="H13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I13">
         <v>9</v>
@@ -55432,7 +55432,7 @@
         <v>9</v>
       </c>
       <c r="H14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I14">
         <v>9</v>
@@ -55468,7 +55468,7 @@
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U14">
         <v>8</v>
@@ -55509,7 +55509,7 @@
         <v>5</v>
       </c>
       <c r="H15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I15">
         <v>5</v>
@@ -55545,7 +55545,7 @@
         <v>-1</v>
       </c>
       <c r="T15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U15">
         <v>5</v>
@@ -55586,7 +55586,7 @@
         <v>7</v>
       </c>
       <c r="H16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I16">
         <v>8</v>
@@ -55663,7 +55663,7 @@
         <v>8</v>
       </c>
       <c r="H17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I17">
         <v>9</v>
@@ -55740,7 +55740,7 @@
         <v>5</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I18">
         <v>6</v>
@@ -55817,7 +55817,7 @@
         <v>9</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I19">
         <v>8</v>
@@ -55894,7 +55894,7 @@
         <v>8</v>
       </c>
       <c r="H20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I20">
         <v>8</v>
@@ -55971,7 +55971,7 @@
         <v>7</v>
       </c>
       <c r="H21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I21">
         <v>6</v>
@@ -56048,7 +56048,7 @@
         <v>4</v>
       </c>
       <c r="H22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I22">
         <v>6</v>
@@ -56084,7 +56084,7 @@
         <v>-1</v>
       </c>
       <c r="T22">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U22">
         <v>5</v>
@@ -56125,7 +56125,7 @@
         <v>7</v>
       </c>
       <c r="H23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I23">
         <v>6</v>
@@ -56202,7 +56202,7 @@
         <v>8</v>
       </c>
       <c r="H24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I24">
         <v>7</v>
@@ -56279,7 +56279,7 @@
         <v>8</v>
       </c>
       <c r="H25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I25">
         <v>8</v>
@@ -56315,7 +56315,7 @@
         <v>-1</v>
       </c>
       <c r="T25">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U25">
         <v>8</v>
@@ -56356,7 +56356,7 @@
         <v>6</v>
       </c>
       <c r="H26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I26">
         <v>7</v>
@@ -56421,7 +56421,7 @@
         <v>7</v>
       </c>
       <c r="H27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I27">
         <v>8</v>
@@ -56462,7 +56462,7 @@
         <v>9</v>
       </c>
       <c r="H28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I28">
         <v>9</v>
@@ -56498,7 +56498,7 @@
         <v>-1</v>
       </c>
       <c r="T28">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U28">
         <v>9</v>
@@ -63957,7 +63957,7 @@
         <v>10</v>
       </c>
       <c r="O4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P4">
         <v>-1</v>
@@ -64046,7 +64046,7 @@
         <v>5</v>
       </c>
       <c r="O5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P5">
         <v>-1</v>
@@ -64088,7 +64088,7 @@
         <v>7</v>
       </c>
       <c r="AC5">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:29">
@@ -64135,7 +64135,7 @@
         <v>10</v>
       </c>
       <c r="O6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P6">
         <v>-1</v>
@@ -64224,7 +64224,7 @@
         <v>5</v>
       </c>
       <c r="O7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P7">
         <v>-1</v>
@@ -64313,7 +64313,7 @@
         <v>6</v>
       </c>
       <c r="O8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P8">
         <v>-1</v>
@@ -64355,7 +64355,7 @@
         <v>8</v>
       </c>
       <c r="AC8">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:29">
@@ -64402,7 +64402,7 @@
         <v>10</v>
       </c>
       <c r="O9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P9">
         <v>-1</v>
@@ -64491,7 +64491,7 @@
         <v>10</v>
       </c>
       <c r="O10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P10">
         <v>-1</v>
@@ -64580,7 +64580,7 @@
         <v>8</v>
       </c>
       <c r="O11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P11">
         <v>-1</v>
@@ -64669,7 +64669,7 @@
         <v>10</v>
       </c>
       <c r="O12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P12">
         <v>-1</v>
@@ -64758,7 +64758,7 @@
         <v>6</v>
       </c>
       <c r="O13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P13">
         <v>-1</v>
@@ -64800,7 +64800,7 @@
         <v>8</v>
       </c>
       <c r="AC13">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:29">
@@ -64847,7 +64847,7 @@
         <v>10</v>
       </c>
       <c r="O14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P14">
         <v>-1</v>
@@ -64889,7 +64889,7 @@
         <v>10</v>
       </c>
       <c r="AC14">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:29">
@@ -64936,7 +64936,7 @@
         <v>5</v>
       </c>
       <c r="O15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P15">
         <v>-1</v>
@@ -64978,7 +64978,7 @@
         <v>7</v>
       </c>
       <c r="AC15">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:29">
@@ -65025,7 +65025,7 @@
         <v>5</v>
       </c>
       <c r="O16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P16">
         <v>-1</v>
@@ -65067,7 +65067,7 @@
         <v>7</v>
       </c>
       <c r="AC16">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17" spans="1:29">
@@ -65114,7 +65114,7 @@
         <v>5</v>
       </c>
       <c r="O17">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P17">
         <v>-1</v>
@@ -65203,7 +65203,7 @@
         <v>10</v>
       </c>
       <c r="O18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P18">
         <v>-1</v>
@@ -65245,7 +65245,7 @@
         <v>10</v>
       </c>
       <c r="AC18">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:29">
@@ -65292,7 +65292,7 @@
         <v>10</v>
       </c>
       <c r="O19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P19">
         <v>-1</v>
@@ -65381,7 +65381,7 @@
         <v>5</v>
       </c>
       <c r="O20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P20">
         <v>-1</v>
@@ -65423,7 +65423,7 @@
         <v>7</v>
       </c>
       <c r="AC20">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:29">
@@ -65470,7 +65470,7 @@
         <v>10</v>
       </c>
       <c r="O21">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P21">
         <v>-1</v>
@@ -65512,7 +65512,7 @@
         <v>10</v>
       </c>
       <c r="AC21">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="22" spans="1:29">
@@ -65559,7 +65559,7 @@
         <v>6</v>
       </c>
       <c r="O22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P22">
         <v>-1</v>
@@ -65601,7 +65601,7 @@
         <v>8</v>
       </c>
       <c r="AC22">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23" spans="1:29">
@@ -65648,7 +65648,7 @@
         <v>10</v>
       </c>
       <c r="O23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P23">
         <v>-1</v>
@@ -65690,7 +65690,7 @@
         <v>10</v>
       </c>
       <c r="AC23">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:29">
@@ -65737,7 +65737,7 @@
         <v>9</v>
       </c>
       <c r="O24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P24">
         <v>-1</v>
@@ -65826,7 +65826,7 @@
         <v>5</v>
       </c>
       <c r="O25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P25">
         <v>-1</v>
@@ -65915,7 +65915,7 @@
         <v>6</v>
       </c>
       <c r="O26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P26">
         <v>-1</v>
@@ -65957,7 +65957,7 @@
         <v>7</v>
       </c>
       <c r="AC26">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:29">
@@ -66004,7 +66004,7 @@
         <v>10</v>
       </c>
       <c r="O27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P27">
         <v>-1</v>
@@ -66093,7 +66093,7 @@
         <v>8</v>
       </c>
       <c r="O28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P28">
         <v>-1</v>
@@ -66182,7 +66182,7 @@
         <v>10</v>
       </c>
       <c r="O29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P29">
         <v>-1</v>
@@ -66271,7 +66271,7 @@
         <v>10</v>
       </c>
       <c r="O30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P30">
         <v>-1</v>
@@ -66360,7 +66360,7 @@
         <v>9</v>
       </c>
       <c r="O31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P31">
         <v>-1</v>
@@ -66449,7 +66449,7 @@
         <v>5</v>
       </c>
       <c r="O32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P32">
         <v>-1</v>
@@ -66491,7 +66491,7 @@
         <v>8</v>
       </c>
       <c r="AC32">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:29">
@@ -66538,7 +66538,7 @@
         <v>5</v>
       </c>
       <c r="O33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P33">
         <v>-1</v>
@@ -66580,7 +66580,7 @@
         <v>8</v>
       </c>
       <c r="AC33">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:29">
@@ -66627,7 +66627,7 @@
         <v>5</v>
       </c>
       <c r="O34">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P34">
         <v>-1</v>
@@ -66669,7 +66669,7 @@
         <v>7</v>
       </c>
       <c r="AC34">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:29">
@@ -66716,7 +66716,7 @@
         <v>10</v>
       </c>
       <c r="O35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P35">
         <v>-1</v>
@@ -66805,7 +66805,7 @@
         <v>10</v>
       </c>
       <c r="O36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P36">
         <v>-1</v>
@@ -66894,7 +66894,7 @@
         <v>5</v>
       </c>
       <c r="O37">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P37">
         <v>-1</v>
@@ -68031,7 +68031,7 @@
         <v>5</v>
       </c>
       <c r="K16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -68067,7 +68067,7 @@
         <v>5</v>
       </c>
       <c r="W16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X16">
         <v>7</v>
@@ -69032,7 +69032,7 @@
         <v>6</v>
       </c>
       <c r="K29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L29">
         <v>9</v>
@@ -69068,7 +69068,7 @@
         <v>5</v>
       </c>
       <c r="W29">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X29">
         <v>9</v>
@@ -69494,7 +69494,7 @@
         <v>6</v>
       </c>
       <c r="K35">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L35">
         <v>5</v>
@@ -69530,7 +69530,7 @@
         <v>5</v>
       </c>
       <c r="W35">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X35">
         <v>5</v>
@@ -69784,7 +69784,7 @@
         <v>10</v>
       </c>
       <c r="K4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L4">
         <v>10</v>
@@ -69861,7 +69861,7 @@
         <v>6</v>
       </c>
       <c r="K5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -69897,7 +69897,7 @@
         <v>5</v>
       </c>
       <c r="W5">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X5">
         <v>5</v>
@@ -69938,7 +69938,7 @@
         <v>8</v>
       </c>
       <c r="K6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L6">
         <v>6</v>
@@ -70015,7 +70015,7 @@
         <v>9</v>
       </c>
       <c r="K7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L7">
         <v>10</v>
@@ -70092,7 +70092,7 @@
         <v>5</v>
       </c>
       <c r="K8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L8">
         <v>0</v>
@@ -70169,7 +70169,7 @@
         <v>8</v>
       </c>
       <c r="K9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="L9">
         <v>10</v>
@@ -70246,7 +70246,7 @@
         <v>8</v>
       </c>
       <c r="K10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L10">
         <v>10</v>
@@ -70323,7 +70323,7 @@
         <v>5</v>
       </c>
       <c r="K11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="L11">
         <v>6</v>
@@ -70359,7 +70359,7 @@
         <v>5</v>
       </c>
       <c r="W11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X11">
         <v>8</v>
@@ -70400,7 +70400,7 @@
         <v>7</v>
       </c>
       <c r="K12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L12">
         <v>6</v>
@@ -70477,7 +70477,7 @@
         <v>10</v>
       </c>
       <c r="K13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L13">
         <v>8</v>
@@ -70513,7 +70513,7 @@
         <v>9</v>
       </c>
       <c r="W13">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X13">
         <v>8</v>
@@ -70554,7 +70554,7 @@
         <v>7</v>
       </c>
       <c r="K14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L14">
         <v>3</v>
@@ -70590,7 +70590,7 @@
         <v>6</v>
       </c>
       <c r="W14">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X14">
         <v>5</v>
@@ -70631,7 +70631,7 @@
         <v>7</v>
       </c>
       <c r="K15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L15">
         <v>3</v>
@@ -70667,7 +70667,7 @@
         <v>7</v>
       </c>
       <c r="W15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="X15">
         <v>5</v>
@@ -70708,7 +70708,7 @@
         <v>9</v>
       </c>
       <c r="K16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="L16">
         <v>3</v>
@@ -70785,7 +70785,7 @@
         <v>5</v>
       </c>
       <c r="K17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="L17">
         <v>3</v>
@@ -70862,7 +70862,7 @@
         <v>9</v>
       </c>
       <c r="K18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L18">
         <v>8</v>
@@ -70939,7 +70939,7 @@
         <v>9</v>
       </c>
       <c r="K19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="L19">
         <v>3</v>
@@ -70998,7 +70998,7 @@
         <v>5</v>
       </c>
       <c r="K20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="O20">
         <v>-1</v>
@@ -78119,7 +78119,7 @@
         <v>7</v>
       </c>
       <c r="O4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P4">
         <v>-1</v>
@@ -78161,7 +78161,7 @@
         <v>6</v>
       </c>
       <c r="AC4">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:29">
@@ -78208,7 +78208,7 @@
         <v>10</v>
       </c>
       <c r="O5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P5">
         <v>-1</v>
@@ -78297,7 +78297,7 @@
         <v>6</v>
       </c>
       <c r="O6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P6">
         <v>-1</v>
@@ -78386,7 +78386,7 @@
         <v>10</v>
       </c>
       <c r="O7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P7">
         <v>-1</v>
@@ -78428,7 +78428,7 @@
         <v>10</v>
       </c>
       <c r="AC7">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:29">
@@ -78475,7 +78475,7 @@
         <v>10</v>
       </c>
       <c r="O8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P8">
         <v>-1</v>
@@ -78564,7 +78564,7 @@
         <v>10</v>
       </c>
       <c r="O9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P9">
         <v>-1</v>
@@ -78653,7 +78653,7 @@
         <v>10</v>
       </c>
       <c r="O10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P10">
         <v>-1</v>
@@ -78695,7 +78695,7 @@
         <v>10</v>
       </c>
       <c r="AC10">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:29">
@@ -78742,7 +78742,7 @@
         <v>5</v>
       </c>
       <c r="O11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P11">
         <v>-1</v>
@@ -78831,7 +78831,7 @@
         <v>5</v>
       </c>
       <c r="O12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P12">
         <v>-1</v>
@@ -78920,7 +78920,7 @@
         <v>10</v>
       </c>
       <c r="O13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P13">
         <v>-1</v>
@@ -79009,7 +79009,7 @@
         <v>9</v>
       </c>
       <c r="O14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P14">
         <v>-1</v>
@@ -79098,7 +79098,7 @@
         <v>10</v>
       </c>
       <c r="O15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P15">
         <v>-1</v>
@@ -79187,7 +79187,7 @@
         <v>10</v>
       </c>
       <c r="O16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P16">
         <v>-1</v>
@@ -79229,7 +79229,7 @@
         <v>10</v>
       </c>
       <c r="AC16">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:29">
@@ -79276,7 +79276,7 @@
         <v>10</v>
       </c>
       <c r="O17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P17">
         <v>-1</v>
@@ -79365,7 +79365,7 @@
         <v>10</v>
       </c>
       <c r="O18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P18">
         <v>-1</v>
@@ -79407,7 +79407,7 @@
         <v>10</v>
       </c>
       <c r="AC18">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:29">
@@ -79454,7 +79454,7 @@
         <v>10</v>
       </c>
       <c r="O19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P19">
         <v>-1</v>
@@ -79496,7 +79496,7 @@
         <v>10</v>
       </c>
       <c r="AC19">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20" spans="1:29">
@@ -79543,7 +79543,7 @@
         <v>10</v>
       </c>
       <c r="O20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P20">
         <v>-1</v>
@@ -79632,7 +79632,7 @@
         <v>9</v>
       </c>
       <c r="O21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P21">
         <v>-1</v>
@@ -79721,7 +79721,7 @@
         <v>10</v>
       </c>
       <c r="O22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P22">
         <v>-1</v>
@@ -79763,7 +79763,7 @@
         <v>10</v>
       </c>
       <c r="AC22">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:29">
@@ -79810,7 +79810,7 @@
         <v>10</v>
       </c>
       <c r="O23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P23">
         <v>-1</v>
@@ -79852,7 +79852,7 @@
         <v>10</v>
       </c>
       <c r="AC23">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" spans="1:29">
@@ -79899,7 +79899,7 @@
         <v>10</v>
       </c>
       <c r="O24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P24">
         <v>-1</v>
@@ -79988,7 +79988,7 @@
         <v>5</v>
       </c>
       <c r="O25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P25">
         <v>-1</v>
@@ -80077,7 +80077,7 @@
         <v>10</v>
       </c>
       <c r="O26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P26">
         <v>-1</v>
@@ -80119,7 +80119,7 @@
         <v>10</v>
       </c>
       <c r="AC26">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:29">
@@ -80166,7 +80166,7 @@
         <v>10</v>
       </c>
       <c r="O27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P27">
         <v>-1</v>
@@ -80255,7 +80255,7 @@
         <v>9</v>
       </c>
       <c r="O28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P28">
         <v>-1</v>
@@ -80297,7 +80297,7 @@
         <v>10</v>
       </c>
       <c r="AC28">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29" spans="1:29">
@@ -80344,7 +80344,7 @@
         <v>10</v>
       </c>
       <c r="O29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P29">
         <v>-1</v>
@@ -80433,7 +80433,7 @@
         <v>10</v>
       </c>
       <c r="O30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P30">
         <v>-1</v>
@@ -80475,7 +80475,7 @@
         <v>10</v>
       </c>
       <c r="AC30">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:29">
@@ -80522,7 +80522,7 @@
         <v>9</v>
       </c>
       <c r="O31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P31">
         <v>-1</v>
@@ -80611,7 +80611,7 @@
         <v>9</v>
       </c>
       <c r="O32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P32">
         <v>-1</v>
@@ -80700,7 +80700,7 @@
         <v>9</v>
       </c>
       <c r="O33">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P33">
         <v>-1</v>
@@ -80742,7 +80742,7 @@
         <v>10</v>
       </c>
       <c r="AC33">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:29">
@@ -80789,7 +80789,7 @@
         <v>10</v>
       </c>
       <c r="O34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P34">
         <v>-1</v>
@@ -80878,7 +80878,7 @@
         <v>8</v>
       </c>
       <c r="O35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P35">
         <v>-1</v>
@@ -80920,7 +80920,7 @@
         <v>9</v>
       </c>
       <c r="AC35">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:29">
@@ -80967,7 +80967,7 @@
         <v>10</v>
       </c>
       <c r="O36">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P36">
         <v>-1</v>
@@ -81009,7 +81009,7 @@
         <v>10</v>
       </c>
       <c r="AC36">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="37" spans="1:29">
@@ -81056,7 +81056,7 @@
         <v>10</v>
       </c>
       <c r="O37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P37">
         <v>-1</v>
@@ -81145,7 +81145,7 @@
         <v>5</v>
       </c>
       <c r="O38">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P38">
         <v>-1</v>
@@ -81234,7 +81234,7 @@
         <v>6</v>
       </c>
       <c r="O39">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P39">
         <v>-1</v>
@@ -81276,7 +81276,7 @@
         <v>8</v>
       </c>
       <c r="AC39">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:29">
@@ -81323,7 +81323,7 @@
         <v>10</v>
       </c>
       <c r="O40">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P40">
         <v>-1</v>
@@ -81412,7 +81412,7 @@
         <v>10</v>
       </c>
       <c r="O41">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P41">
         <v>-1</v>
@@ -81501,7 +81501,7 @@
         <v>9</v>
       </c>
       <c r="O42">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P42">
         <v>-1</v>
@@ -81742,7 +81742,7 @@
         <v>8</v>
       </c>
       <c r="O4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P4">
         <v>-1</v>
@@ -81784,7 +81784,7 @@
         <v>8</v>
       </c>
       <c r="AC4">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:29">
@@ -81831,7 +81831,7 @@
         <v>10</v>
       </c>
       <c r="O5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P5">
         <v>-1</v>
@@ -81873,7 +81873,7 @@
         <v>10</v>
       </c>
       <c r="AC5">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:29">
@@ -81920,7 +81920,7 @@
         <v>10</v>
       </c>
       <c r="O6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P6">
         <v>-1</v>
@@ -82009,7 +82009,7 @@
         <v>10</v>
       </c>
       <c r="O7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P7">
         <v>-1</v>
@@ -82051,7 +82051,7 @@
         <v>10</v>
       </c>
       <c r="AC7">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:29">
@@ -82098,7 +82098,7 @@
         <v>8</v>
       </c>
       <c r="O8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P8">
         <v>-1</v>
@@ -82140,7 +82140,7 @@
         <v>9</v>
       </c>
       <c r="AC8">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:29">
@@ -82187,7 +82187,7 @@
         <v>5</v>
       </c>
       <c r="O9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P9">
         <v>-1</v>
@@ -82229,7 +82229,7 @@
         <v>8</v>
       </c>
       <c r="AC9">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:29">
@@ -82276,7 +82276,7 @@
         <v>9</v>
       </c>
       <c r="O10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P10">
         <v>-1</v>
@@ -82318,7 +82318,7 @@
         <v>10</v>
       </c>
       <c r="AC10">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:29">
@@ -82365,7 +82365,7 @@
         <v>10</v>
       </c>
       <c r="O11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P11">
         <v>-1</v>
@@ -82407,7 +82407,7 @@
         <v>10</v>
       </c>
       <c r="AC11">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:29">
@@ -82454,7 +82454,7 @@
         <v>5</v>
       </c>
       <c r="O12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P12">
         <v>-1</v>
@@ -82543,7 +82543,7 @@
         <v>8</v>
       </c>
       <c r="O13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P13">
         <v>-1</v>
@@ -82585,7 +82585,7 @@
         <v>9</v>
       </c>
       <c r="AC13">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:29">
@@ -82632,7 +82632,7 @@
         <v>8</v>
       </c>
       <c r="O14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P14">
         <v>-1</v>
@@ -82721,7 +82721,7 @@
         <v>8</v>
       </c>
       <c r="O15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P15">
         <v>-1</v>
@@ -82810,7 +82810,7 @@
         <v>7</v>
       </c>
       <c r="O16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P16">
         <v>-1</v>
@@ -82899,7 +82899,7 @@
         <v>10</v>
       </c>
       <c r="O17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P17">
         <v>-1</v>
@@ -82941,7 +82941,7 @@
         <v>10</v>
       </c>
       <c r="AC17">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18" spans="1:29">
@@ -82988,7 +82988,7 @@
         <v>8</v>
       </c>
       <c r="O18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P18">
         <v>-1</v>
@@ -83077,7 +83077,7 @@
         <v>8</v>
       </c>
       <c r="O19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P19">
         <v>-1</v>
@@ -83166,7 +83166,7 @@
         <v>8</v>
       </c>
       <c r="O20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P20">
         <v>-1</v>
@@ -83208,7 +83208,7 @@
         <v>9</v>
       </c>
       <c r="AC20">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21" spans="1:29">
@@ -83255,7 +83255,7 @@
         <v>9</v>
       </c>
       <c r="O21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P21">
         <v>-1</v>
@@ -83297,7 +83297,7 @@
         <v>10</v>
       </c>
       <c r="AC21">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:29">
@@ -83344,7 +83344,7 @@
         <v>10</v>
       </c>
       <c r="O22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="P22">
         <v>-1</v>
@@ -83433,7 +83433,7 @@
         <v>5</v>
       </c>
       <c r="O23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P23">
         <v>-1</v>
@@ -83522,7 +83522,7 @@
         <v>8</v>
       </c>
       <c r="O24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P24">
         <v>-1</v>
@@ -83611,7 +83611,7 @@
         <v>7</v>
       </c>
       <c r="O25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P25">
         <v>-1</v>
@@ -83653,7 +83653,7 @@
         <v>8</v>
       </c>
       <c r="AC25">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:29">
@@ -83700,7 +83700,7 @@
         <v>8</v>
       </c>
       <c r="O26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="P26">
         <v>-1</v>
@@ -83742,7 +83742,7 @@
         <v>9</v>
       </c>
       <c r="AC26">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:29">
@@ -83789,7 +83789,7 @@
         <v>7</v>
       </c>
       <c r="O27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P27">
         <v>-1</v>
@@ -83831,7 +83831,7 @@
         <v>9</v>
       </c>
       <c r="AC27">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:29">
@@ -83878,7 +83878,7 @@
         <v>10</v>
       </c>
       <c r="O28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P28">
         <v>-1</v>
@@ -83967,7 +83967,7 @@
         <v>10</v>
       </c>
       <c r="O29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P29">
         <v>-1</v>
@@ -84009,7 +84009,7 @@
         <v>10</v>
       </c>
       <c r="AC29">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30" spans="1:29">
@@ -84056,7 +84056,7 @@
         <v>7</v>
       </c>
       <c r="O30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P30">
         <v>-1</v>
@@ -84145,7 +84145,7 @@
         <v>5</v>
       </c>
       <c r="O31">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="P31">
         <v>-1</v>
@@ -84234,7 +84234,7 @@
         <v>7</v>
       </c>
       <c r="O32">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P32">
         <v>-1</v>
@@ -84276,7 +84276,7 @@
         <v>8</v>
       </c>
       <c r="AC32">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="33" spans="1:29">
@@ -84323,7 +84323,7 @@
         <v>6</v>
       </c>
       <c r="O33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="P33">
         <v>-1</v>
@@ -84365,7 +84365,7 @@
         <v>7</v>
       </c>
       <c r="AC33">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -84527,7 +84527,7 @@
         <v>10</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I4">
         <v>9</v>
@@ -84604,7 +84604,7 @@
         <v>9</v>
       </c>
       <c r="H5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I5">
         <v>9</v>
@@ -84681,7 +84681,7 @@
         <v>10</v>
       </c>
       <c r="H6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I6">
         <v>9</v>
@@ -84717,7 +84717,7 @@
         <v>-1</v>
       </c>
       <c r="T6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U6">
         <v>8</v>
@@ -84758,7 +84758,7 @@
         <v>9</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I7">
         <v>9</v>
@@ -84794,7 +84794,7 @@
         <v>-1</v>
       </c>
       <c r="T7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U7">
         <v>9</v>
@@ -84835,7 +84835,7 @@
         <v>9</v>
       </c>
       <c r="H8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I8">
         <v>9</v>
@@ -84912,7 +84912,7 @@
         <v>8</v>
       </c>
       <c r="H9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I9">
         <v>9</v>
@@ -84989,7 +84989,7 @@
         <v>9</v>
       </c>
       <c r="H10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I10">
         <v>9</v>
@@ -85025,7 +85025,7 @@
         <v>-1</v>
       </c>
       <c r="T10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U10">
         <v>7</v>
@@ -85066,7 +85066,7 @@
         <v>8</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I11">
         <v>9</v>
@@ -85143,7 +85143,7 @@
         <v>10</v>
       </c>
       <c r="H12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I12">
         <v>9</v>
@@ -85179,7 +85179,7 @@
         <v>-1</v>
       </c>
       <c r="T12">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U12">
         <v>8</v>
@@ -85220,7 +85220,7 @@
         <v>8</v>
       </c>
       <c r="H13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I13">
         <v>9</v>
@@ -85297,7 +85297,7 @@
         <v>9</v>
       </c>
       <c r="H14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I14">
         <v>9</v>
@@ -85333,7 +85333,7 @@
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U14">
         <v>8</v>
@@ -85374,7 +85374,7 @@
         <v>7</v>
       </c>
       <c r="H15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I15">
         <v>9</v>
@@ -85451,7 +85451,7 @@
         <v>10</v>
       </c>
       <c r="H16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I16">
         <v>9</v>
@@ -85528,7 +85528,7 @@
         <v>10</v>
       </c>
       <c r="H17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I17">
         <v>9</v>
@@ -85564,7 +85564,7 @@
         <v>-1</v>
       </c>
       <c r="T17">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U17">
         <v>8</v>
@@ -85605,7 +85605,7 @@
         <v>6</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I18">
         <v>9</v>
@@ -85641,7 +85641,7 @@
         <v>-1</v>
       </c>
       <c r="T18">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="U18">
         <v>7</v>
@@ -85682,7 +85682,7 @@
         <v>10</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I19">
         <v>9</v>
@@ -85718,7 +85718,7 @@
         <v>-1</v>
       </c>
       <c r="T19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U19">
         <v>9</v>
@@ -85759,7 +85759,7 @@
         <v>10</v>
       </c>
       <c r="H20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I20">
         <v>9</v>
@@ -85795,7 +85795,7 @@
         <v>-1</v>
       </c>
       <c r="T20">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U20">
         <v>8</v>
@@ -85836,7 +85836,7 @@
         <v>9</v>
       </c>
       <c r="H21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I21">
         <v>9</v>
@@ -85913,7 +85913,7 @@
         <v>9</v>
       </c>
       <c r="H22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I22">
         <v>9</v>
@@ -85990,7 +85990,7 @@
         <v>8</v>
       </c>
       <c r="H23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I23">
         <v>9</v>
@@ -86067,7 +86067,7 @@
         <v>10</v>
       </c>
       <c r="H24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I24">
         <v>9</v>
@@ -86144,7 +86144,7 @@
         <v>9</v>
       </c>
       <c r="H25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I25">
         <v>9</v>
@@ -86215,7 +86215,7 @@
         <v>5</v>
       </c>
       <c r="H26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="K26">
         <v>6</v>
@@ -86274,7 +86274,7 @@
         <v>10</v>
       </c>
       <c r="H27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I27">
         <v>9</v>
@@ -86351,7 +86351,7 @@
         <v>10</v>
       </c>
       <c r="H28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I28">
         <v>9</v>
@@ -86428,7 +86428,7 @@
         <v>9</v>
       </c>
       <c r="H29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I29">
         <v>9</v>
@@ -86505,7 +86505,7 @@
         <v>9</v>
       </c>
       <c r="H30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I30">
         <v>9</v>
@@ -86541,7 +86541,7 @@
         <v>-1</v>
       </c>
       <c r="T30">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U30">
         <v>8</v>
@@ -86582,7 +86582,7 @@
         <v>10</v>
       </c>
       <c r="H31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I31">
         <v>9</v>
@@ -86618,7 +86618,7 @@
         <v>-1</v>
       </c>
       <c r="T31">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U31">
         <v>9</v>
@@ -86659,7 +86659,7 @@
         <v>10</v>
       </c>
       <c r="H32">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I32">
         <v>9</v>
@@ -86736,7 +86736,7 @@
         <v>8</v>
       </c>
       <c r="H33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I33">
         <v>9</v>
@@ -86949,7 +86949,7 @@
         <v>9</v>
       </c>
       <c r="H4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I4">
         <v>8</v>
@@ -86985,7 +86985,7 @@
         <v>-1</v>
       </c>
       <c r="T4">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U4">
         <v>7</v>
@@ -87026,7 +87026,7 @@
         <v>9</v>
       </c>
       <c r="H5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I5">
         <v>9</v>
@@ -87103,7 +87103,7 @@
         <v>9</v>
       </c>
       <c r="H6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I6">
         <v>7</v>
@@ -87180,7 +87180,7 @@
         <v>6</v>
       </c>
       <c r="H7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I7">
         <v>9</v>
@@ -87216,7 +87216,7 @@
         <v>-1</v>
       </c>
       <c r="T7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U7">
         <v>9</v>
@@ -87257,7 +87257,7 @@
         <v>9</v>
       </c>
       <c r="H8">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I8">
         <v>7</v>
@@ -87334,7 +87334,7 @@
         <v>8</v>
       </c>
       <c r="H9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I9">
         <v>9</v>
@@ -87370,7 +87370,7 @@
         <v>-1</v>
       </c>
       <c r="T9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U9">
         <v>9</v>
@@ -87411,7 +87411,7 @@
         <v>9</v>
       </c>
       <c r="H10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I10">
         <v>10</v>
@@ -87488,7 +87488,7 @@
         <v>8</v>
       </c>
       <c r="H11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I11">
         <v>8</v>
@@ -87524,7 +87524,7 @@
         <v>-1</v>
       </c>
       <c r="T11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U11">
         <v>7</v>
@@ -87565,7 +87565,7 @@
         <v>9</v>
       </c>
       <c r="H12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I12">
         <v>10</v>
@@ -87601,7 +87601,7 @@
         <v>-1</v>
       </c>
       <c r="T12">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U12">
         <v>9</v>
@@ -87642,7 +87642,7 @@
         <v>9</v>
       </c>
       <c r="H13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I13">
         <v>8</v>
@@ -87678,7 +87678,7 @@
         <v>-1</v>
       </c>
       <c r="T13">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U13">
         <v>8</v>
@@ -87719,7 +87719,7 @@
         <v>9</v>
       </c>
       <c r="H14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I14">
         <v>8</v>
@@ -87755,7 +87755,7 @@
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U14">
         <v>8</v>
@@ -87796,7 +87796,7 @@
         <v>9</v>
       </c>
       <c r="H15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I15">
         <v>9</v>
@@ -87873,7 +87873,7 @@
         <v>9</v>
       </c>
       <c r="H16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I16">
         <v>7</v>
@@ -87950,7 +87950,7 @@
         <v>8</v>
       </c>
       <c r="H17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I17">
         <v>9</v>
@@ -87986,7 +87986,7 @@
         <v>-1</v>
       </c>
       <c r="T17">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U17">
         <v>9</v>
@@ -88027,7 +88027,7 @@
         <v>8</v>
       </c>
       <c r="H18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I18">
         <v>10</v>
@@ -88063,7 +88063,7 @@
         <v>-1</v>
       </c>
       <c r="T18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U18">
         <v>9</v>
@@ -88104,7 +88104,7 @@
         <v>6</v>
       </c>
       <c r="H19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I19">
         <v>5</v>
@@ -88181,7 +88181,7 @@
         <v>9</v>
       </c>
       <c r="H20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I20">
         <v>9</v>
@@ -88217,7 +88217,7 @@
         <v>-1</v>
       </c>
       <c r="T20">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U20">
         <v>8</v>
@@ -88258,7 +88258,7 @@
         <v>7</v>
       </c>
       <c r="H21">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I21">
         <v>7</v>
@@ -88294,7 +88294,7 @@
         <v>-1</v>
       </c>
       <c r="T21">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U21">
         <v>7</v>
@@ -88335,7 +88335,7 @@
         <v>9</v>
       </c>
       <c r="H22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I22">
         <v>10</v>
@@ -88412,7 +88412,7 @@
         <v>5</v>
       </c>
       <c r="H23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="I23">
         <v>5</v>
@@ -88489,7 +88489,7 @@
         <v>7</v>
       </c>
       <c r="H24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I24">
         <v>8</v>
@@ -88525,7 +88525,7 @@
         <v>-1</v>
       </c>
       <c r="T24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U24">
         <v>7</v>
@@ -88566,7 +88566,7 @@
         <v>10</v>
       </c>
       <c r="H25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I25">
         <v>8</v>
@@ -88643,7 +88643,7 @@
         <v>8</v>
       </c>
       <c r="H26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I26">
         <v>9</v>
@@ -88679,7 +88679,7 @@
         <v>-1</v>
       </c>
       <c r="T26">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U26">
         <v>8</v>
@@ -88720,7 +88720,7 @@
         <v>5</v>
       </c>
       <c r="H27">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="I27">
         <v>5</v>
@@ -88756,7 +88756,7 @@
         <v>-1</v>
       </c>
       <c r="T27">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U27">
         <v>5</v>
@@ -88797,7 +88797,7 @@
         <v>9</v>
       </c>
       <c r="H28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I28">
         <v>9</v>
@@ -88874,7 +88874,7 @@
         <v>8</v>
       </c>
       <c r="H29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I29">
         <v>9</v>
@@ -88910,7 +88910,7 @@
         <v>-1</v>
       </c>
       <c r="T29">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U29">
         <v>8</v>
@@ -88951,7 +88951,7 @@
         <v>5</v>
       </c>
       <c r="H30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="I30">
         <v>6</v>
@@ -89028,7 +89028,7 @@
         <v>9</v>
       </c>
       <c r="H31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I31">
         <v>9</v>
@@ -89105,7 +89105,7 @@
         <v>9</v>
       </c>
       <c r="H32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I32">
         <v>9</v>
@@ -89141,7 +89141,7 @@
         <v>-1</v>
       </c>
       <c r="T32">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U32">
         <v>9</v>
@@ -89182,7 +89182,7 @@
         <v>9</v>
       </c>
       <c r="H33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I33">
         <v>9</v>
@@ -89218,7 +89218,7 @@
         <v>-1</v>
       </c>
       <c r="T33">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U33">
         <v>9</v>
@@ -89259,7 +89259,7 @@
         <v>8</v>
       </c>
       <c r="H34">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I34">
         <v>7</v>
@@ -89336,7 +89336,7 @@
         <v>7</v>
       </c>
       <c r="H35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I35">
         <v>8</v>
@@ -89413,7 +89413,7 @@
         <v>9</v>
       </c>
       <c r="H36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="I36">
         <v>9</v>
@@ -89490,7 +89490,7 @@
         <v>5</v>
       </c>
       <c r="H37">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="I37">
         <v>7</v>
@@ -89567,7 +89567,7 @@
         <v>10</v>
       </c>
       <c r="H38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I38">
         <v>9</v>
@@ -89644,7 +89644,7 @@
         <v>9</v>
       </c>
       <c r="H39">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I39">
         <v>10</v>
@@ -89721,7 +89721,7 @@
         <v>9</v>
       </c>
       <c r="H40">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I40">
         <v>8</v>
@@ -89798,7 +89798,7 @@
         <v>10</v>
       </c>
       <c r="H41">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I41">
         <v>8</v>
@@ -89875,7 +89875,7 @@
         <v>8</v>
       </c>
       <c r="H42">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I42">
         <v>8</v>
@@ -89911,7 +89911,7 @@
         <v>-1</v>
       </c>
       <c r="T42">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U42">
         <v>7</v>
@@ -89952,7 +89952,7 @@
         <v>8</v>
       </c>
       <c r="H43">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I43">
         <v>9</v>
@@ -89988,7 +89988,7 @@
         <v>-1</v>
       </c>
       <c r="T43">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U43">
         <v>8</v>
@@ -90029,7 +90029,7 @@
         <v>9</v>
       </c>
       <c r="H44">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I44">
         <v>9</v>
@@ -90106,7 +90106,7 @@
         <v>10</v>
       </c>
       <c r="H45">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="I45">
         <v>9</v>

</xml_diff>

<commit_message>
Estadisticos Segundo Parcial 20231
</commit_message>
<xml_diff>
--- a/Calificaciones20231.xlsx
+++ b/Calificaciones20231.xlsx
@@ -34817,7 +34817,7 @@
         <v>4</v>
       </c>
       <c r="I4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J4">
         <v>5</v>
@@ -34906,7 +34906,7 @@
         <v>4</v>
       </c>
       <c r="I5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J5">
         <v>7</v>
@@ -34948,7 +34948,7 @@
         <v>-1</v>
       </c>
       <c r="W5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X5">
         <v>6</v>
@@ -34995,7 +34995,7 @@
         <v>9</v>
       </c>
       <c r="I6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J6">
         <v>7</v>
@@ -35084,7 +35084,7 @@
         <v>8</v>
       </c>
       <c r="I7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J7">
         <v>5</v>
@@ -35126,7 +35126,7 @@
         <v>-1</v>
       </c>
       <c r="W7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X7">
         <v>5</v>
@@ -35173,7 +35173,7 @@
         <v>7</v>
       </c>
       <c r="I8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J8">
         <v>5</v>
@@ -35215,7 +35215,7 @@
         <v>-1</v>
       </c>
       <c r="W8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X8">
         <v>5</v>
@@ -35262,7 +35262,7 @@
         <v>10</v>
       </c>
       <c r="I9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J9">
         <v>8</v>
@@ -35351,7 +35351,7 @@
         <v>8</v>
       </c>
       <c r="I10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J10">
         <v>6</v>
@@ -35393,7 +35393,7 @@
         <v>-1</v>
       </c>
       <c r="W10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X10">
         <v>5</v>
@@ -35440,7 +35440,7 @@
         <v>7</v>
       </c>
       <c r="I11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J11">
         <v>6</v>
@@ -35482,7 +35482,7 @@
         <v>-1</v>
       </c>
       <c r="W11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X11">
         <v>5</v>
@@ -35529,7 +35529,7 @@
         <v>9</v>
       </c>
       <c r="I12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J12">
         <v>6</v>
@@ -35571,7 +35571,7 @@
         <v>-1</v>
       </c>
       <c r="W12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X12">
         <v>7</v>
@@ -35618,7 +35618,7 @@
         <v>9</v>
       </c>
       <c r="I13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J13">
         <v>7</v>
@@ -35707,7 +35707,7 @@
         <v>6</v>
       </c>
       <c r="I14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J14">
         <v>5</v>
@@ -35796,7 +35796,7 @@
         <v>5</v>
       </c>
       <c r="I15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J15">
         <v>5</v>
@@ -35838,7 +35838,7 @@
         <v>-1</v>
       </c>
       <c r="W15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X15">
         <v>5</v>
@@ -35885,7 +35885,7 @@
         <v>6</v>
       </c>
       <c r="I16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J16">
         <v>7</v>
@@ -35974,7 +35974,7 @@
         <v>6</v>
       </c>
       <c r="I17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="J17">
         <v>5</v>
@@ -36063,7 +36063,7 @@
         <v>7</v>
       </c>
       <c r="I18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J18">
         <v>7</v>
@@ -36105,7 +36105,7 @@
         <v>-1</v>
       </c>
       <c r="W18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X18">
         <v>6</v>
@@ -36152,7 +36152,7 @@
         <v>9</v>
       </c>
       <c r="I19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J19">
         <v>7</v>
@@ -36241,7 +36241,7 @@
         <v>10</v>
       </c>
       <c r="I20">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="J20">
         <v>8</v>
@@ -36330,7 +36330,7 @@
         <v>10</v>
       </c>
       <c r="I21">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J21">
         <v>9</v>
@@ -36372,7 +36372,7 @@
         <v>-1</v>
       </c>
       <c r="W21">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X21">
         <v>9</v>
@@ -36419,7 +36419,7 @@
         <v>6</v>
       </c>
       <c r="I22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J22">
         <v>7</v>
@@ -36461,7 +36461,7 @@
         <v>-1</v>
       </c>
       <c r="W22">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X22">
         <v>6</v>
@@ -36508,7 +36508,7 @@
         <v>10</v>
       </c>
       <c r="I23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="J23">
         <v>8</v>
@@ -36550,7 +36550,7 @@
         <v>-1</v>
       </c>
       <c r="W23">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X23">
         <v>8</v>
@@ -36597,7 +36597,7 @@
         <v>4</v>
       </c>
       <c r="I24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J24">
         <v>5</v>
@@ -36639,7 +36639,7 @@
         <v>-1</v>
       </c>
       <c r="W24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X24">
         <v>5</v>
@@ -36686,7 +36686,7 @@
         <v>10</v>
       </c>
       <c r="I25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="J25">
         <v>8</v>
@@ -36775,7 +36775,7 @@
         <v>9</v>
       </c>
       <c r="I26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="J26">
         <v>6</v>
@@ -36817,7 +36817,7 @@
         <v>-1</v>
       </c>
       <c r="W26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X26">
         <v>5</v>
@@ -36864,7 +36864,7 @@
         <v>8</v>
       </c>
       <c r="I27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="J27">
         <v>5</v>
@@ -36906,7 +36906,7 @@
         <v>-1</v>
       </c>
       <c r="W27">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X27">
         <v>6</v>
@@ -51929,7 +51929,7 @@
         <v>8</v>
       </c>
       <c r="L8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M8">
         <v>5</v>
@@ -51965,7 +51965,7 @@
         <v>8</v>
       </c>
       <c r="X8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Y8">
         <v>7</v>
@@ -52006,7 +52006,7 @@
         <v>7</v>
       </c>
       <c r="L9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M9">
         <v>5</v>
@@ -52042,7 +52042,7 @@
         <v>7</v>
       </c>
       <c r="X9">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y9">
         <v>7</v>
@@ -52083,7 +52083,7 @@
         <v>7</v>
       </c>
       <c r="L10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M10">
         <v>9</v>
@@ -52119,7 +52119,7 @@
         <v>8</v>
       </c>
       <c r="X10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Y10">
         <v>10</v>
@@ -52160,7 +52160,7 @@
         <v>5</v>
       </c>
       <c r="L11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M11">
         <v>5</v>
@@ -52314,7 +52314,7 @@
         <v>7</v>
       </c>
       <c r="L13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M13">
         <v>5</v>
@@ -52350,7 +52350,7 @@
         <v>7</v>
       </c>
       <c r="X13">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y13">
         <v>5</v>
@@ -52468,7 +52468,7 @@
         <v>5</v>
       </c>
       <c r="L15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M15">
         <v>5</v>
@@ -52504,7 +52504,7 @@
         <v>5</v>
       </c>
       <c r="X15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y15">
         <v>5</v>
@@ -52622,7 +52622,7 @@
         <v>7</v>
       </c>
       <c r="L17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M17">
         <v>5</v>
@@ -53007,7 +53007,7 @@
         <v>7</v>
       </c>
       <c r="L22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M22">
         <v>5</v>
@@ -53161,7 +53161,7 @@
         <v>7</v>
       </c>
       <c r="L24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M24">
         <v>5</v>
@@ -53267,7 +53267,7 @@
         <v>7</v>
       </c>
       <c r="L26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="M26">
         <v>6</v>
@@ -53303,7 +53303,7 @@
         <v>7</v>
       </c>
       <c r="X26">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y26">
         <v>6</v>
@@ -53344,7 +53344,7 @@
         <v>8</v>
       </c>
       <c r="L27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M27">
         <v>7</v>
@@ -53380,7 +53380,7 @@
         <v>7</v>
       </c>
       <c r="X27">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="Y27">
         <v>7</v>
@@ -53421,7 +53421,7 @@
         <v>8</v>
       </c>
       <c r="L28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M28">
         <v>8</v>
@@ -53457,7 +53457,7 @@
         <v>8</v>
       </c>
       <c r="X28">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Y28">
         <v>9</v>
@@ -53498,7 +53498,7 @@
         <v>8</v>
       </c>
       <c r="L29">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M29">
         <v>6</v>
@@ -53575,7 +53575,7 @@
         <v>5</v>
       </c>
       <c r="L30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M30">
         <v>5</v>
@@ -53611,7 +53611,7 @@
         <v>5</v>
       </c>
       <c r="X30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y30">
         <v>5</v>
@@ -53652,7 +53652,7 @@
         <v>8</v>
       </c>
       <c r="L31">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M31">
         <v>8</v>
@@ -53688,7 +53688,7 @@
         <v>8</v>
       </c>
       <c r="X31">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="Y31">
         <v>9</v>
@@ -53758,7 +53758,7 @@
         <v>6</v>
       </c>
       <c r="L33">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M33">
         <v>5</v>
@@ -53835,7 +53835,7 @@
         <v>5</v>
       </c>
       <c r="L34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M34">
         <v>5</v>
@@ -53871,7 +53871,7 @@
         <v>6</v>
       </c>
       <c r="X34">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Y34">
         <v>5</v>
@@ -53912,7 +53912,7 @@
         <v>6</v>
       </c>
       <c r="L35">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M35">
         <v>10</v>
@@ -53948,7 +53948,7 @@
         <v>5</v>
       </c>
       <c r="X35">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Y35">
         <v>9</v>
@@ -53989,7 +53989,7 @@
         <v>10</v>
       </c>
       <c r="L36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="M36">
         <v>7</v>
@@ -54095,7 +54095,7 @@
         <v>7</v>
       </c>
       <c r="L38">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M38">
         <v>6</v>
@@ -54131,7 +54131,7 @@
         <v>8</v>
       </c>
       <c r="X38">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y38">
         <v>6</v>
@@ -54172,7 +54172,7 @@
         <v>7</v>
       </c>
       <c r="L39">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M39">
         <v>7</v>
@@ -54278,7 +54278,7 @@
         <v>7</v>
       </c>
       <c r="L41">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M41">
         <v>5</v>
@@ -54355,7 +54355,7 @@
         <v>6</v>
       </c>
       <c r="L42">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M42">
         <v>5</v>
@@ -54391,7 +54391,7 @@
         <v>6</v>
       </c>
       <c r="X42">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y42">
         <v>6</v>
@@ -54461,7 +54461,7 @@
         <v>7</v>
       </c>
       <c r="L44">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M44">
         <v>5</v>
@@ -54497,7 +54497,7 @@
         <v>7</v>
       </c>
       <c r="X44">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y44">
         <v>6</v>
@@ -69944,7 +69944,7 @@
         <v>6</v>
       </c>
       <c r="M6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -69980,7 +69980,7 @@
         <v>6</v>
       </c>
       <c r="Y6">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:25">

</xml_diff>

<commit_message>
Estadisticos Segundo Parcial Milka
</commit_message>
<xml_diff>
--- a/Calificaciones20231.xlsx
+++ b/Calificaciones20231.xlsx
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2084" uniqueCount="1080">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2085" uniqueCount="1081">
   <si>
     <t>Materia</t>
   </si>
@@ -3259,6 +3259,9 @@
   </si>
   <si>
     <t>FLORES MIXCOHA CRISTHIAN ALFONSO</t>
+  </si>
+  <si>
+    <t>GUTIERREZ FLORES MILKA SARAY</t>
   </si>
   <si>
     <t>HERNANDEZ ILLESCAS REDA ALAN</t>
@@ -4164,7 +4167,7 @@
         <v>7</v>
       </c>
       <c r="I8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J8">
         <v>7</v>
@@ -4206,7 +4209,7 @@
         <v>-1</v>
       </c>
       <c r="W8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X8">
         <v>7</v>
@@ -7268,7 +7271,7 @@
         <v>8</v>
       </c>
       <c r="H16">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I16">
         <v>6</v>
@@ -7304,7 +7307,7 @@
         <v>-1</v>
       </c>
       <c r="T16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="U16">
         <v>7</v>
@@ -10975,7 +10978,7 @@
         <v>9</v>
       </c>
       <c r="H19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I19">
         <v>9</v>
@@ -11011,7 +11014,7 @@
         <v>-1</v>
       </c>
       <c r="T19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U19">
         <v>8</v>
@@ -11976,7 +11979,7 @@
         <v>5</v>
       </c>
       <c r="H32">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="I32">
         <v>9</v>
@@ -12012,7 +12015,7 @@
         <v>-1</v>
       </c>
       <c r="T32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U32">
         <v>7</v>
@@ -15510,7 +15513,7 @@
         <v>5</v>
       </c>
       <c r="L4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M4">
         <v>9</v>
@@ -15572,7 +15575,7 @@
         <v>7</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D5">
         <v>8</v>
@@ -15599,7 +15602,7 @@
         <v>10</v>
       </c>
       <c r="L5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M5">
         <v>9</v>
@@ -15635,13 +15638,13 @@
         <v>7</v>
       </c>
       <c r="X5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y5">
         <v>9</v>
       </c>
       <c r="Z5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA5">
         <v>7</v>
@@ -15688,7 +15691,7 @@
         <v>10</v>
       </c>
       <c r="L6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M6">
         <v>10</v>
@@ -15730,7 +15733,7 @@
         <v>10</v>
       </c>
       <c r="Z6">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AA6">
         <v>10</v>
@@ -15777,7 +15780,7 @@
         <v>6</v>
       </c>
       <c r="L7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M7">
         <v>8</v>
@@ -15819,7 +15822,7 @@
         <v>7</v>
       </c>
       <c r="Z7">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA7">
         <v>9</v>
@@ -15866,7 +15869,7 @@
         <v>9</v>
       </c>
       <c r="L8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M8">
         <v>8</v>
@@ -15908,7 +15911,7 @@
         <v>9</v>
       </c>
       <c r="Z8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AA8">
         <v>9</v>
@@ -16044,7 +16047,7 @@
         <v>9</v>
       </c>
       <c r="L10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M10">
         <v>8</v>
@@ -16086,7 +16089,7 @@
         <v>8</v>
       </c>
       <c r="Z10">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AA10">
         <v>9</v>
@@ -16133,7 +16136,7 @@
         <v>9</v>
       </c>
       <c r="L11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M11">
         <v>9</v>
@@ -16175,7 +16178,7 @@
         <v>9</v>
       </c>
       <c r="Z11">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AA11">
         <v>9</v>
@@ -16222,7 +16225,7 @@
         <v>8</v>
       </c>
       <c r="L12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M12">
         <v>9</v>
@@ -16264,7 +16267,7 @@
         <v>9</v>
       </c>
       <c r="Z12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA12">
         <v>9</v>
@@ -16400,7 +16403,7 @@
         <v>8</v>
       </c>
       <c r="L14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M14">
         <v>8</v>
@@ -16442,7 +16445,7 @@
         <v>8</v>
       </c>
       <c r="Z14">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AA14">
         <v>9</v>
@@ -16489,7 +16492,7 @@
         <v>5</v>
       </c>
       <c r="L15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M15">
         <v>8</v>
@@ -16531,7 +16534,7 @@
         <v>8</v>
       </c>
       <c r="Z15">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA15">
         <v>9</v>
@@ -16551,7 +16554,7 @@
         <v>6</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D16">
         <v>7</v>
@@ -16578,7 +16581,7 @@
         <v>9</v>
       </c>
       <c r="L16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M16">
         <v>7</v>
@@ -16614,7 +16617,7 @@
         <v>6</v>
       </c>
       <c r="X16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y16">
         <v>8</v>
@@ -16640,7 +16643,7 @@
         <v>8</v>
       </c>
       <c r="C17">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D17">
         <v>7</v>
@@ -16667,7 +16670,7 @@
         <v>8</v>
       </c>
       <c r="L17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M17">
         <v>5</v>
@@ -16703,7 +16706,7 @@
         <v>7</v>
       </c>
       <c r="X17">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y17">
         <v>8</v>
@@ -16756,7 +16759,7 @@
         <v>6</v>
       </c>
       <c r="L18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M18">
         <v>9</v>
@@ -16798,7 +16801,7 @@
         <v>8</v>
       </c>
       <c r="Z18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA18">
         <v>9</v>
@@ -16845,7 +16848,7 @@
         <v>5</v>
       </c>
       <c r="L19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M19">
         <v>5</v>
@@ -16934,7 +16937,7 @@
         <v>5</v>
       </c>
       <c r="L20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M20">
         <v>5</v>
@@ -16976,7 +16979,7 @@
         <v>5</v>
       </c>
       <c r="Z20">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA20">
         <v>7</v>
@@ -17023,7 +17026,7 @@
         <v>9</v>
       </c>
       <c r="L21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M21">
         <v>10</v>
@@ -17065,7 +17068,7 @@
         <v>8</v>
       </c>
       <c r="Z21">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA21">
         <v>10</v>
@@ -17112,7 +17115,7 @@
         <v>9</v>
       </c>
       <c r="L22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M22">
         <v>9</v>
@@ -17154,7 +17157,7 @@
         <v>8</v>
       </c>
       <c r="Z22">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA22">
         <v>10</v>
@@ -17201,7 +17204,7 @@
         <v>8</v>
       </c>
       <c r="L23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M23">
         <v>7</v>
@@ -17243,7 +17246,7 @@
         <v>8</v>
       </c>
       <c r="Z23">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA23">
         <v>8</v>
@@ -17263,7 +17266,7 @@
         <v>7</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D24">
         <v>7</v>
@@ -17290,7 +17293,7 @@
         <v>6</v>
       </c>
       <c r="L24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M24">
         <v>5</v>
@@ -17326,7 +17329,7 @@
         <v>7</v>
       </c>
       <c r="X24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y24">
         <v>7</v>
@@ -17352,7 +17355,7 @@
         <v>5</v>
       </c>
       <c r="C25">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D25">
         <v>8</v>
@@ -17379,7 +17382,7 @@
         <v>7</v>
       </c>
       <c r="L25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="M25">
         <v>6</v>
@@ -17415,13 +17418,13 @@
         <v>5</v>
       </c>
       <c r="X25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y25">
         <v>8</v>
       </c>
       <c r="Z25">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA25">
         <v>7</v>
@@ -17468,7 +17471,7 @@
         <v>9</v>
       </c>
       <c r="L26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M26">
         <v>8</v>
@@ -17510,7 +17513,7 @@
         <v>9</v>
       </c>
       <c r="Z26">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA26">
         <v>9</v>
@@ -17557,7 +17560,7 @@
         <v>8</v>
       </c>
       <c r="L27">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="M27">
         <v>10</v>
@@ -17599,7 +17602,7 @@
         <v>9</v>
       </c>
       <c r="Z27">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AA27">
         <v>10</v>
@@ -17646,7 +17649,7 @@
         <v>9</v>
       </c>
       <c r="L28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M28">
         <v>6</v>
@@ -17735,7 +17738,7 @@
         <v>9</v>
       </c>
       <c r="L29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M29">
         <v>7</v>
@@ -17777,7 +17780,7 @@
         <v>9</v>
       </c>
       <c r="Z29">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA29">
         <v>9</v>
@@ -17797,7 +17800,7 @@
         <v>5</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D30">
         <v>9</v>
@@ -17824,7 +17827,7 @@
         <v>5</v>
       </c>
       <c r="L30">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="M30">
         <v>6</v>
@@ -17860,13 +17863,13 @@
         <v>5</v>
       </c>
       <c r="X30">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="Y30">
         <v>7</v>
       </c>
       <c r="Z30">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA30">
         <v>8</v>
@@ -17913,7 +17916,7 @@
         <v>9</v>
       </c>
       <c r="L31">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M31">
         <v>10</v>
@@ -17955,7 +17958,7 @@
         <v>9</v>
       </c>
       <c r="Z31">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AA31">
         <v>10</v>
@@ -18002,7 +18005,7 @@
         <v>9</v>
       </c>
       <c r="L32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M32">
         <v>7</v>
@@ -18044,7 +18047,7 @@
         <v>9</v>
       </c>
       <c r="Z32">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA32">
         <v>9</v>
@@ -18091,7 +18094,7 @@
         <v>9</v>
       </c>
       <c r="L33">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M33">
         <v>10</v>
@@ -18133,7 +18136,7 @@
         <v>9</v>
       </c>
       <c r="Z33">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AA33">
         <v>10</v>
@@ -18369,7 +18372,7 @@
         <v>10</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E5">
         <v>6</v>
@@ -18423,7 +18426,7 @@
         <v>9</v>
       </c>
       <c r="V5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W5">
         <v>6</v>
@@ -18831,7 +18834,7 @@
         <v>7</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E11">
         <v>6</v>
@@ -18885,7 +18888,7 @@
         <v>7</v>
       </c>
       <c r="V11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W11">
         <v>7</v>
@@ -26307,7 +26310,7 @@
         <v>6</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -26370,7 +26373,7 @@
         <v>8</v>
       </c>
       <c r="X8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y8">
         <v>7</v>
@@ -26841,7 +26844,7 @@
         <v>6</v>
       </c>
       <c r="C14">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D14">
         <v>7</v>
@@ -26904,7 +26907,7 @@
         <v>8</v>
       </c>
       <c r="X14">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y14">
         <v>6</v>
@@ -27185,7 +27188,7 @@
         <v>5</v>
       </c>
       <c r="C18">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D18">
         <v>5</v>
@@ -27274,7 +27277,7 @@
         <v>6</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D19">
         <v>8</v>
@@ -27452,7 +27455,7 @@
         <v>6</v>
       </c>
       <c r="C21">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D21">
         <v>8</v>
@@ -27515,7 +27518,7 @@
         <v>8</v>
       </c>
       <c r="X21">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y21">
         <v>8</v>
@@ -27719,7 +27722,7 @@
         <v>9</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D24">
         <v>6</v>
@@ -27782,7 +27785,7 @@
         <v>9</v>
       </c>
       <c r="X24">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y24">
         <v>7</v>
@@ -28253,7 +28256,7 @@
         <v>8</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D30">
         <v>8</v>
@@ -28316,7 +28319,7 @@
         <v>9</v>
       </c>
       <c r="X30">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y30">
         <v>8</v>
@@ -29215,7 +29218,7 @@
         <v>10</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E13">
         <v>4</v>
@@ -29269,7 +29272,7 @@
         <v>10</v>
       </c>
       <c r="V13">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W13">
         <v>6</v>
@@ -29908,7 +29911,7 @@
         <v>8</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E22">
         <v>4</v>
@@ -29962,7 +29965,7 @@
         <v>8</v>
       </c>
       <c r="V22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W22">
         <v>5</v>
@@ -30755,7 +30758,7 @@
         <v>7</v>
       </c>
       <c r="D33">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E33">
         <v>6</v>
@@ -30809,7 +30812,7 @@
         <v>7</v>
       </c>
       <c r="V33">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W33">
         <v>7</v>
@@ -30832,7 +30835,7 @@
         <v>7</v>
       </c>
       <c r="D34">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E34">
         <v>4</v>
@@ -30886,7 +30889,7 @@
         <v>7</v>
       </c>
       <c r="V34">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W34">
         <v>5</v>
@@ -30909,7 +30912,7 @@
         <v>8</v>
       </c>
       <c r="D35">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E35">
         <v>6</v>
@@ -30963,7 +30966,7 @@
         <v>8</v>
       </c>
       <c r="V35">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W35">
         <v>7</v>
@@ -31063,7 +31066,7 @@
         <v>6</v>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E37">
         <v>4</v>
@@ -31117,7 +31120,7 @@
         <v>6</v>
       </c>
       <c r="V37">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W37">
         <v>5</v>
@@ -51778,7 +51781,7 @@
         <v>9</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N6">
         <v>-1</v>
@@ -51814,7 +51817,7 @@
         <v>9</v>
       </c>
       <c r="Y6">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -51932,7 +51935,7 @@
         <v>8</v>
       </c>
       <c r="M8">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -51968,7 +51971,7 @@
         <v>9</v>
       </c>
       <c r="Y8">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -53915,7 +53918,7 @@
         <v>5</v>
       </c>
       <c r="M35">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="N35">
         <v>-1</v>
@@ -53951,7 +53954,7 @@
         <v>6</v>
       </c>
       <c r="Y35">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:25">
@@ -53992,7 +53995,7 @@
         <v>9</v>
       </c>
       <c r="M36">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="N36">
         <v>-1</v>
@@ -54028,7 +54031,7 @@
         <v>10</v>
       </c>
       <c r="Y36">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="37" spans="1:25">
@@ -54098,7 +54101,7 @@
         <v>7</v>
       </c>
       <c r="M38">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N38">
         <v>-1</v>
@@ -54134,7 +54137,7 @@
         <v>7</v>
       </c>
       <c r="Y38">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:25">
@@ -58383,7 +58386,7 @@
         <v>10</v>
       </c>
       <c r="G27">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H27">
         <v>10</v>
@@ -58437,7 +58440,7 @@
         <v>10</v>
       </c>
       <c r="Y27">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:25">
@@ -73164,7 +73167,7 @@
 
 <file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y15"/>
+  <dimension ref="A1:Y16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" customWidth="1"/>
@@ -73523,40 +73526,40 @@
         <v>1071</v>
       </c>
       <c r="B7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D7">
-        <v>7</v>
+        <v>-1</v>
       </c>
       <c r="E7">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F7">
-        <v>10</v>
+        <v>-1</v>
       </c>
       <c r="G7">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H7">
         <v>9</v>
       </c>
       <c r="I7">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J7">
-        <v>8</v>
+        <v>-1</v>
       </c>
       <c r="K7">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L7">
-        <v>7</v>
+        <v>-1</v>
       </c>
       <c r="M7">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="N7">
         <v>-1</v>
@@ -73580,19 +73583,19 @@
         <v>9</v>
       </c>
       <c r="U7">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="V7">
-        <v>8</v>
+        <v>-1</v>
       </c>
       <c r="W7">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="X7">
-        <v>9</v>
+        <v>-1</v>
       </c>
       <c r="Y7">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -73600,40 +73603,40 @@
         <v>1072</v>
       </c>
       <c r="B8">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E8">
         <v>9</v>
       </c>
       <c r="F8">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G8">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H8">
         <v>9</v>
       </c>
       <c r="I8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K8">
         <v>10</v>
       </c>
       <c r="L8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="N8">
         <v>-1</v>
@@ -73654,22 +73657,22 @@
         <v>-1</v>
       </c>
       <c r="T8">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="U8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="V8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="W8">
         <v>10</v>
       </c>
       <c r="X8">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="Y8">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -73677,13 +73680,13 @@
         <v>1073</v>
       </c>
       <c r="B9">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C9">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E9">
         <v>9</v>
@@ -73692,7 +73695,7 @@
         <v>6</v>
       </c>
       <c r="G9">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H9">
         <v>9</v>
@@ -73707,7 +73710,7 @@
         <v>10</v>
       </c>
       <c r="L9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M9">
         <v>9</v>
@@ -73731,22 +73734,22 @@
         <v>-1</v>
       </c>
       <c r="T9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="W9">
         <v>10</v>
       </c>
       <c r="X9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Y9">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -73754,40 +73757,40 @@
         <v>1074</v>
       </c>
       <c r="B10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10">
         <v>9</v>
       </c>
       <c r="F10">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I10">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J10">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K10">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L10">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N10">
         <v>-1</v>
@@ -73808,22 +73811,22 @@
         <v>-1</v>
       </c>
       <c r="T10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="U10">
         <v>9</v>
       </c>
       <c r="V10">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="W10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="X10">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Y10">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -73834,37 +73837,37 @@
         <v>5</v>
       </c>
       <c r="C11">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D11">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E11">
         <v>9</v>
       </c>
       <c r="F11">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G11">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I11">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J11">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L11">
         <v>5</v>
       </c>
       <c r="M11">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N11">
         <v>-1</v>
@@ -73888,19 +73891,19 @@
         <v>7</v>
       </c>
       <c r="U11">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="V11">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="W11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X11">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Y11">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -73908,7 +73911,7 @@
         <v>1076</v>
       </c>
       <c r="B12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12">
         <v>7</v>
@@ -73920,28 +73923,28 @@
         <v>9</v>
       </c>
       <c r="F12">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G12">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H12">
         <v>9</v>
       </c>
       <c r="I12">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J12">
         <v>6</v>
       </c>
       <c r="K12">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L12">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M12">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="N12">
         <v>-1</v>
@@ -73965,19 +73968,19 @@
         <v>7</v>
       </c>
       <c r="U12">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V12">
         <v>5</v>
       </c>
       <c r="W12">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="X12">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="Y12">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -73988,19 +73991,19 @@
         <v>4</v>
       </c>
       <c r="C13">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D13">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E13">
         <v>9</v>
       </c>
       <c r="F13">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H13">
         <v>9</v>
@@ -74009,7 +74012,7 @@
         <v>8</v>
       </c>
       <c r="J13">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="K13">
         <v>10</v>
@@ -74018,7 +74021,7 @@
         <v>6</v>
       </c>
       <c r="M13">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="N13">
         <v>-1</v>
@@ -74042,19 +74045,19 @@
         <v>7</v>
       </c>
       <c r="U13">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="V13">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="W13">
         <v>10</v>
       </c>
       <c r="X13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Y13">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -74062,40 +74065,40 @@
         <v>1078</v>
       </c>
       <c r="B14">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C14">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D14">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E14">
         <v>9</v>
       </c>
       <c r="F14">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G14">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H14">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I14">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J14">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K14">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M14">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N14">
         <v>-1</v>
@@ -74116,22 +74119,22 @@
         <v>-1</v>
       </c>
       <c r="T14">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="U14">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="V14">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="W14">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="X14">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Y14">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -74142,37 +74145,37 @@
         <v>5</v>
       </c>
       <c r="C15">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D15">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E15">
         <v>9</v>
       </c>
       <c r="F15">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G15">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H15">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I15">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J15">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K15">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M15">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N15">
         <v>-1</v>
@@ -74193,21 +74196,98 @@
         <v>-1</v>
       </c>
       <c r="T15">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="U15">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="V15">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W15">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="X15">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Y15">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25">
+      <c r="A16" s="1" t="s">
+        <v>1080</v>
+      </c>
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16">
+        <v>8</v>
+      </c>
+      <c r="D16">
+        <v>7</v>
+      </c>
+      <c r="E16">
+        <v>9</v>
+      </c>
+      <c r="F16">
+        <v>9</v>
+      </c>
+      <c r="G16">
+        <v>9</v>
+      </c>
+      <c r="H16">
+        <v>8</v>
+      </c>
+      <c r="I16">
+        <v>10</v>
+      </c>
+      <c r="J16">
+        <v>8</v>
+      </c>
+      <c r="K16">
+        <v>10</v>
+      </c>
+      <c r="L16">
+        <v>6</v>
+      </c>
+      <c r="M16">
+        <v>10</v>
+      </c>
+      <c r="N16">
+        <v>-1</v>
+      </c>
+      <c r="O16">
+        <v>-1</v>
+      </c>
+      <c r="P16">
+        <v>-1</v>
+      </c>
+      <c r="Q16">
+        <v>-1</v>
+      </c>
+      <c r="R16">
+        <v>-1</v>
+      </c>
+      <c r="S16">
+        <v>-1</v>
+      </c>
+      <c r="T16">
+        <v>7</v>
+      </c>
+      <c r="U16">
+        <v>9</v>
+      </c>
+      <c r="V16">
+        <v>8</v>
+      </c>
+      <c r="W16">
+        <v>10</v>
+      </c>
+      <c r="X16">
+        <v>8</v>
+      </c>
+      <c r="Y16">
         <v>10</v>
       </c>
     </row>
@@ -76807,7 +76887,7 @@
         <v>5</v>
       </c>
       <c r="N31">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="O31">
         <v>6</v>
@@ -76849,7 +76929,7 @@
         <v>5</v>
       </c>
       <c r="AB31">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="AC31">
         <v>7</v>
@@ -76964,7 +77044,7 @@
         <v>6</v>
       </c>
       <c r="G33">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="H33">
         <v>5</v>
@@ -76985,7 +77065,7 @@
         <v>5</v>
       </c>
       <c r="N33">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="O33">
         <v>5</v>
@@ -77027,7 +77107,7 @@
         <v>5</v>
       </c>
       <c r="AB33">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="AC33">
         <v>5</v>
@@ -86659,7 +86739,7 @@
         <v>10</v>
       </c>
       <c r="H32">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I32">
         <v>9</v>
@@ -86695,7 +86775,7 @@
         <v>-1</v>
       </c>
       <c r="T32">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="U32">
         <v>10</v>

</xml_diff>

<commit_message>
Estadisticos Tercer Parcial 8
</commit_message>
<xml_diff>
--- a/Calificaciones20231.xlsx
+++ b/Calificaciones20231.xlsx
@@ -21396,7 +21396,7 @@
         <v>7</v>
       </c>
       <c r="Q4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="R4">
         <v>7</v>
@@ -31485,7 +31485,7 @@
         <v>5</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q4">
         <v>5</v>
@@ -31500,7 +31500,7 @@
         <v>5</v>
       </c>
       <c r="U4">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="V4">
         <v>-1</v>
@@ -31521,7 +31521,7 @@
         <v>5</v>
       </c>
       <c r="AB4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AC4">
         <v>5</v>
@@ -31574,7 +31574,7 @@
         <v>5</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q5">
         <v>5</v>
@@ -31589,7 +31589,7 @@
         <v>5</v>
       </c>
       <c r="U5">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="V5">
         <v>-1</v>
@@ -31663,7 +31663,7 @@
         <v>5</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q6">
         <v>8</v>
@@ -31678,7 +31678,7 @@
         <v>10</v>
       </c>
       <c r="U6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V6">
         <v>-1</v>
@@ -31699,7 +31699,7 @@
         <v>10</v>
       </c>
       <c r="AB6">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AC6">
         <v>6</v>
@@ -31752,7 +31752,7 @@
         <v>6</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q7">
         <v>8</v>
@@ -31767,13 +31767,13 @@
         <v>7</v>
       </c>
       <c r="U7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V7">
         <v>-1</v>
       </c>
       <c r="W7">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X7">
         <v>7</v>
@@ -31841,7 +31841,7 @@
         <v>6</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q8">
         <v>5</v>
@@ -31856,13 +31856,13 @@
         <v>9</v>
       </c>
       <c r="U8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V8">
         <v>-1</v>
       </c>
       <c r="W8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X8">
         <v>6</v>
@@ -31877,7 +31877,7 @@
         <v>7</v>
       </c>
       <c r="AB8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AC8">
         <v>6</v>
@@ -31930,7 +31930,7 @@
         <v>5</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q9">
         <v>7</v>
@@ -31945,7 +31945,7 @@
         <v>5</v>
       </c>
       <c r="U9">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="V9">
         <v>-1</v>
@@ -32019,7 +32019,7 @@
         <v>6</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q10">
         <v>8</v>
@@ -32034,7 +32034,7 @@
         <v>10</v>
       </c>
       <c r="U10">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V10">
         <v>-1</v>
@@ -32108,7 +32108,7 @@
         <v>5</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q11">
         <v>6</v>
@@ -32123,7 +32123,7 @@
         <v>7</v>
       </c>
       <c r="U11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V11">
         <v>-1</v>
@@ -32197,7 +32197,7 @@
         <v>6</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q12">
         <v>6</v>
@@ -32212,7 +32212,7 @@
         <v>5</v>
       </c>
       <c r="U12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V12">
         <v>-1</v>
@@ -32233,7 +32233,7 @@
         <v>6</v>
       </c>
       <c r="AB12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC12">
         <v>7</v>
@@ -32286,7 +32286,7 @@
         <v>6</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q13">
         <v>7</v>
@@ -32301,7 +32301,7 @@
         <v>8</v>
       </c>
       <c r="U13">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V13">
         <v>-1</v>
@@ -32322,7 +32322,7 @@
         <v>6</v>
       </c>
       <c r="AB13">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AC13">
         <v>7</v>
@@ -32375,7 +32375,7 @@
         <v>6</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q14">
         <v>8</v>
@@ -32390,7 +32390,7 @@
         <v>10</v>
       </c>
       <c r="U14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V14">
         <v>-1</v>
@@ -32464,7 +32464,7 @@
         <v>5</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q15">
         <v>5</v>
@@ -32479,7 +32479,7 @@
         <v>5</v>
       </c>
       <c r="U15">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="V15">
         <v>-1</v>
@@ -32553,7 +32553,7 @@
         <v>5</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q16">
         <v>7</v>
@@ -32568,7 +32568,7 @@
         <v>8</v>
       </c>
       <c r="U16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V16">
         <v>-1</v>
@@ -32589,7 +32589,7 @@
         <v>6</v>
       </c>
       <c r="AB16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC16">
         <v>5</v>
@@ -32642,7 +32642,7 @@
         <v>5</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q17">
         <v>7</v>
@@ -32657,7 +32657,7 @@
         <v>9</v>
       </c>
       <c r="U17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V17">
         <v>-1</v>
@@ -32731,7 +32731,7 @@
         <v>5</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q18">
         <v>7</v>
@@ -32746,7 +32746,7 @@
         <v>5</v>
       </c>
       <c r="U18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V18">
         <v>-1</v>
@@ -32767,7 +32767,7 @@
         <v>5</v>
       </c>
       <c r="AB18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC18">
         <v>5</v>
@@ -32820,7 +32820,7 @@
         <v>5</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q19">
         <v>7</v>
@@ -32835,7 +32835,7 @@
         <v>8</v>
       </c>
       <c r="U19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V19">
         <v>-1</v>
@@ -32856,7 +32856,7 @@
         <v>6</v>
       </c>
       <c r="AB19">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AC19">
         <v>6</v>
@@ -32909,7 +32909,7 @@
         <v>6</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q20">
         <v>7</v>
@@ -32924,7 +32924,7 @@
         <v>9</v>
       </c>
       <c r="U20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V20">
         <v>-1</v>
@@ -32998,7 +32998,7 @@
         <v>5</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q21">
         <v>6</v>
@@ -33013,7 +33013,7 @@
         <v>5</v>
       </c>
       <c r="U21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V21">
         <v>-1</v>
@@ -33087,7 +33087,7 @@
         <v>5</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q22">
         <v>6</v>
@@ -33102,7 +33102,7 @@
         <v>5</v>
       </c>
       <c r="U22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V22">
         <v>-1</v>
@@ -33176,7 +33176,7 @@
         <v>5</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q23">
         <v>7</v>
@@ -33191,7 +33191,7 @@
         <v>8</v>
       </c>
       <c r="U23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V23">
         <v>-1</v>
@@ -33265,7 +33265,7 @@
         <v>5</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q24">
         <v>5</v>
@@ -33280,7 +33280,7 @@
         <v>5</v>
       </c>
       <c r="U24">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="V24">
         <v>-1</v>
@@ -33354,7 +33354,7 @@
         <v>5</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q25">
         <v>6</v>
@@ -33369,7 +33369,7 @@
         <v>5</v>
       </c>
       <c r="U25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V25">
         <v>-1</v>
@@ -33443,7 +33443,7 @@
         <v>5</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q26">
         <v>7</v>
@@ -33458,13 +33458,13 @@
         <v>7</v>
       </c>
       <c r="U26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V26">
         <v>-1</v>
       </c>
       <c r="W26">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X26">
         <v>7</v>
@@ -33532,7 +33532,7 @@
         <v>5</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q27">
         <v>7</v>
@@ -33547,7 +33547,7 @@
         <v>7</v>
       </c>
       <c r="U27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="V27">
         <v>-1</v>
@@ -33568,7 +33568,7 @@
         <v>6</v>
       </c>
       <c r="AB27">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC27">
         <v>6</v>
@@ -33621,7 +33621,7 @@
         <v>5</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q28">
         <v>7</v>
@@ -33636,7 +33636,7 @@
         <v>9</v>
       </c>
       <c r="U28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V28">
         <v>-1</v>
@@ -33710,7 +33710,7 @@
         <v>5</v>
       </c>
       <c r="P29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q29">
         <v>5</v>
@@ -33725,7 +33725,7 @@
         <v>5</v>
       </c>
       <c r="U29">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="V29">
         <v>-1</v>
@@ -33799,7 +33799,7 @@
         <v>6</v>
       </c>
       <c r="P30">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q30">
         <v>8</v>
@@ -33814,13 +33814,13 @@
         <v>8</v>
       </c>
       <c r="U30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V30">
         <v>-1</v>
       </c>
       <c r="W30">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X30">
         <v>8</v>
@@ -33888,7 +33888,7 @@
         <v>5</v>
       </c>
       <c r="P31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q31">
         <v>7</v>
@@ -33903,7 +33903,7 @@
         <v>7</v>
       </c>
       <c r="U31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V31">
         <v>-1</v>
@@ -33924,7 +33924,7 @@
         <v>6</v>
       </c>
       <c r="AB31">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC31">
         <v>5</v>
@@ -33977,7 +33977,7 @@
         <v>5</v>
       </c>
       <c r="P32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q32">
         <v>6</v>
@@ -33992,13 +33992,13 @@
         <v>9</v>
       </c>
       <c r="U32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V32">
         <v>-1</v>
       </c>
       <c r="W32">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X32">
         <v>7</v>
@@ -34013,7 +34013,7 @@
         <v>7</v>
       </c>
       <c r="AB32">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AC32">
         <v>6</v>
@@ -34066,7 +34066,7 @@
         <v>5</v>
       </c>
       <c r="P33">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q33">
         <v>7</v>
@@ -34081,7 +34081,7 @@
         <v>7</v>
       </c>
       <c r="U33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V33">
         <v>-1</v>
@@ -34102,7 +34102,7 @@
         <v>7</v>
       </c>
       <c r="AB33">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AC33">
         <v>6</v>
@@ -34155,7 +34155,7 @@
         <v>5</v>
       </c>
       <c r="P34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q34">
         <v>5</v>
@@ -34170,7 +34170,7 @@
         <v>5</v>
       </c>
       <c r="U34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="V34">
         <v>-1</v>
@@ -34244,7 +34244,7 @@
         <v>6</v>
       </c>
       <c r="P35">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q35">
         <v>7</v>
@@ -34259,7 +34259,7 @@
         <v>7</v>
       </c>
       <c r="U35">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V35">
         <v>-1</v>
@@ -34333,7 +34333,7 @@
         <v>5</v>
       </c>
       <c r="P36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q36">
         <v>7</v>
@@ -34348,7 +34348,7 @@
         <v>8</v>
       </c>
       <c r="U36">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V36">
         <v>-1</v>
@@ -34422,7 +34422,7 @@
         <v>6</v>
       </c>
       <c r="P37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q37">
         <v>7</v>
@@ -34437,7 +34437,7 @@
         <v>9</v>
       </c>
       <c r="U37">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V37">
         <v>-1</v>
@@ -34511,7 +34511,7 @@
         <v>5</v>
       </c>
       <c r="P38">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q38">
         <v>6</v>
@@ -34526,7 +34526,7 @@
         <v>7</v>
       </c>
       <c r="U38">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="V38">
         <v>-1</v>
@@ -34547,7 +34547,7 @@
         <v>6</v>
       </c>
       <c r="AB38">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC38">
         <v>5</v>
@@ -34600,7 +34600,7 @@
         <v>5</v>
       </c>
       <c r="P39">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q39">
         <v>7</v>
@@ -34615,13 +34615,13 @@
         <v>8</v>
       </c>
       <c r="U39">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="V39">
         <v>-1</v>
       </c>
       <c r="W39">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X39">
         <v>7</v>
@@ -34636,7 +34636,7 @@
         <v>6</v>
       </c>
       <c r="AB39">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AC39">
         <v>5</v>
@@ -44375,7 +44375,7 @@
         <v>7</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q4">
         <v>9</v>
@@ -44464,7 +44464,7 @@
         <v>5</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q5">
         <v>5</v>
@@ -44485,7 +44485,7 @@
         <v>7</v>
       </c>
       <c r="W5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X5">
         <v>6</v>
@@ -44553,7 +44553,7 @@
         <v>5</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q6">
         <v>8</v>
@@ -44642,7 +44642,7 @@
         <v>5</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q7">
         <v>7</v>
@@ -44731,7 +44731,7 @@
         <v>6</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q8">
         <v>8</v>
@@ -44752,7 +44752,7 @@
         <v>7</v>
       </c>
       <c r="W8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X8">
         <v>7</v>
@@ -44820,7 +44820,7 @@
         <v>5</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q9">
         <v>7</v>
@@ -44841,7 +44841,7 @@
         <v>6</v>
       </c>
       <c r="W9">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X9">
         <v>7</v>
@@ -44909,7 +44909,7 @@
         <v>5</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q10">
         <v>9</v>
@@ -44930,7 +44930,7 @@
         <v>5</v>
       </c>
       <c r="W10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X10">
         <v>8</v>
@@ -44998,7 +44998,7 @@
         <v>6</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q11">
         <v>7</v>
@@ -45087,7 +45087,7 @@
         <v>5</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q12">
         <v>6</v>
@@ -45176,7 +45176,7 @@
         <v>9</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q13">
         <v>8</v>
@@ -45265,7 +45265,7 @@
         <v>6</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q14">
         <v>5</v>
@@ -45354,7 +45354,7 @@
         <v>6</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q15">
         <v>7</v>
@@ -45443,7 +45443,7 @@
         <v>6</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q16">
         <v>7</v>
@@ -45532,7 +45532,7 @@
         <v>5</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q17">
         <v>5</v>
@@ -45621,7 +45621,7 @@
         <v>5</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q18">
         <v>6</v>
@@ -45642,7 +45642,7 @@
         <v>7</v>
       </c>
       <c r="W18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X18">
         <v>6</v>
@@ -45710,7 +45710,7 @@
         <v>9</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q19">
         <v>8</v>
@@ -45799,7 +45799,7 @@
         <v>5</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q20">
         <v>5</v>
@@ -45888,7 +45888,7 @@
         <v>10</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q21">
         <v>8</v>
@@ -45909,7 +45909,7 @@
         <v>9</v>
       </c>
       <c r="W21">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X21">
         <v>7</v>
@@ -45977,7 +45977,7 @@
         <v>10</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q22">
         <v>10</v>
@@ -45998,7 +45998,7 @@
         <v>9</v>
       </c>
       <c r="W22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="X22">
         <v>9</v>
@@ -46066,7 +46066,7 @@
         <v>10</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q23">
         <v>8</v>
@@ -46155,7 +46155,7 @@
         <v>5</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q24">
         <v>5</v>
@@ -46244,7 +46244,7 @@
         <v>5</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q25">
         <v>5</v>
@@ -46333,7 +46333,7 @@
         <v>5</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q26">
         <v>8</v>
@@ -46422,7 +46422,7 @@
         <v>5</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q27">
         <v>5</v>
@@ -46511,7 +46511,7 @@
         <v>5</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q28">
         <v>5</v>
@@ -46600,7 +46600,7 @@
         <v>5</v>
       </c>
       <c r="P29">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q29">
         <v>7</v>
@@ -46621,7 +46621,7 @@
         <v>5</v>
       </c>
       <c r="W29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X29">
         <v>7</v>
@@ -46689,7 +46689,7 @@
         <v>5</v>
       </c>
       <c r="P30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q30">
         <v>9</v>
@@ -46778,7 +46778,7 @@
         <v>8</v>
       </c>
       <c r="P31">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q31">
         <v>8</v>
@@ -46867,7 +46867,7 @@
         <v>9</v>
       </c>
       <c r="P32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q32">
         <v>7</v>
@@ -46956,7 +46956,7 @@
         <v>8</v>
       </c>
       <c r="P33">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q33">
         <v>7</v>
@@ -47045,7 +47045,7 @@
         <v>8</v>
       </c>
       <c r="P34">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q34">
         <v>8</v>
@@ -47134,7 +47134,7 @@
         <v>5</v>
       </c>
       <c r="P35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q35">
         <v>7</v>
@@ -47223,7 +47223,7 @@
         <v>9</v>
       </c>
       <c r="P36">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q36">
         <v>8</v>
@@ -47244,7 +47244,7 @@
         <v>9</v>
       </c>
       <c r="W36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X36">
         <v>7</v>
@@ -47312,7 +47312,7 @@
         <v>5</v>
       </c>
       <c r="P37">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q37">
         <v>5</v>
@@ -47401,7 +47401,7 @@
         <v>5</v>
       </c>
       <c r="P38">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q38">
         <v>5</v>
@@ -47490,7 +47490,7 @@
         <v>5</v>
       </c>
       <c r="P39">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="Q39">
         <v>4</v>
@@ -47511,7 +47511,7 @@
         <v>5</v>
       </c>
       <c r="W39">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="X39">
         <v>5</v>
@@ -47579,7 +47579,7 @@
         <v>5</v>
       </c>
       <c r="P40">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q40">
         <v>4</v>
@@ -47820,7 +47820,7 @@
         <v>5</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q4">
         <v>7</v>
@@ -47838,7 +47838,7 @@
         <v>6</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W4">
         <v>7</v>
@@ -47909,7 +47909,7 @@
         <v>5</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q5">
         <v>8</v>
@@ -47927,7 +47927,7 @@
         <v>6</v>
       </c>
       <c r="V5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W5">
         <v>6</v>
@@ -47998,7 +47998,7 @@
         <v>6</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q6">
         <v>10</v>
@@ -48016,7 +48016,7 @@
         <v>9</v>
       </c>
       <c r="V6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W6">
         <v>7</v>
@@ -48087,7 +48087,7 @@
         <v>6</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q7">
         <v>10</v>
@@ -48105,7 +48105,7 @@
         <v>10</v>
       </c>
       <c r="V7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W7">
         <v>8</v>
@@ -48126,7 +48126,7 @@
         <v>10</v>
       </c>
       <c r="AC7">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:29">
@@ -48176,7 +48176,7 @@
         <v>5</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q8">
         <v>8</v>
@@ -48194,7 +48194,7 @@
         <v>5</v>
       </c>
       <c r="V8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W8">
         <v>5</v>
@@ -48265,7 +48265,7 @@
         <v>6</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q9">
         <v>10</v>
@@ -48283,10 +48283,10 @@
         <v>8</v>
       </c>
       <c r="V9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X9">
         <v>10</v>
@@ -48354,7 +48354,7 @@
         <v>6</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q10">
         <v>10</v>
@@ -48372,10 +48372,10 @@
         <v>9</v>
       </c>
       <c r="V10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X10">
         <v>10</v>
@@ -48393,7 +48393,7 @@
         <v>9</v>
       </c>
       <c r="AC10">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:29">
@@ -48443,7 +48443,7 @@
         <v>5</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q11">
         <v>5</v>
@@ -48461,7 +48461,7 @@
         <v>5</v>
       </c>
       <c r="V11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W11">
         <v>5</v>
@@ -48532,7 +48532,7 @@
         <v>5</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q12">
         <v>6</v>
@@ -48550,10 +48550,10 @@
         <v>6</v>
       </c>
       <c r="V12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W12">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X12">
         <v>6</v>
@@ -48621,7 +48621,7 @@
         <v>5</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q13">
         <v>8</v>
@@ -48639,7 +48639,7 @@
         <v>9</v>
       </c>
       <c r="V13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W13">
         <v>6</v>
@@ -48660,7 +48660,7 @@
         <v>8</v>
       </c>
       <c r="AC13">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:29">
@@ -48710,7 +48710,7 @@
         <v>6</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q14">
         <v>7</v>
@@ -48728,10 +48728,10 @@
         <v>9</v>
       </c>
       <c r="V14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W14">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X14">
         <v>6</v>
@@ -48799,7 +48799,7 @@
         <v>6</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q15">
         <v>8</v>
@@ -48817,7 +48817,7 @@
         <v>6</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W15">
         <v>6</v>
@@ -48888,7 +48888,7 @@
         <v>6</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q16">
         <v>7</v>
@@ -48906,7 +48906,7 @@
         <v>7</v>
       </c>
       <c r="V16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W16">
         <v>6</v>
@@ -48927,7 +48927,7 @@
         <v>7</v>
       </c>
       <c r="AC16">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:29">
@@ -48977,7 +48977,7 @@
         <v>5</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q17">
         <v>9</v>
@@ -48995,7 +48995,7 @@
         <v>10</v>
       </c>
       <c r="V17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W17">
         <v>7</v>
@@ -49016,7 +49016,7 @@
         <v>10</v>
       </c>
       <c r="AC17">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:29">
@@ -49066,7 +49066,7 @@
         <v>5</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q18">
         <v>8</v>
@@ -49084,7 +49084,7 @@
         <v>5</v>
       </c>
       <c r="V18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W18">
         <v>5</v>
@@ -49105,7 +49105,7 @@
         <v>6</v>
       </c>
       <c r="AC18">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:29">
@@ -49155,7 +49155,7 @@
         <v>5</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q19">
         <v>5</v>
@@ -49173,7 +49173,7 @@
         <v>5</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W19">
         <v>5</v>
@@ -49244,7 +49244,7 @@
         <v>5</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q20">
         <v>5</v>
@@ -49262,7 +49262,7 @@
         <v>5</v>
       </c>
       <c r="V20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W20">
         <v>5</v>
@@ -49333,7 +49333,7 @@
         <v>6</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q21">
         <v>8</v>
@@ -49351,10 +49351,10 @@
         <v>6</v>
       </c>
       <c r="V21">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W21">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X21">
         <v>7</v>
@@ -49422,7 +49422,7 @@
         <v>5</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q22">
         <v>5</v>
@@ -49440,7 +49440,7 @@
         <v>5</v>
       </c>
       <c r="V22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W22">
         <v>5</v>
@@ -61319,16 +61319,16 @@
         <v>7</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R4">
         <v>-1</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T4">
         <v>-1</v>
@@ -61340,16 +61340,16 @@
         <v>-1</v>
       </c>
       <c r="W4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y4">
         <v>7</v>
       </c>
       <c r="Z4">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA4">
         <v>7</v>
@@ -61411,13 +61411,13 @@
         <v>9</v>
       </c>
       <c r="Q5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R5">
         <v>-1</v>
       </c>
       <c r="S5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T5">
         <v>-1</v>
@@ -61432,13 +61432,13 @@
         <v>8</v>
       </c>
       <c r="X5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y5">
         <v>5</v>
       </c>
       <c r="Z5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AA5">
         <v>5</v>
@@ -61500,13 +61500,13 @@
         <v>8</v>
       </c>
       <c r="Q6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="R6">
         <v>-1</v>
       </c>
       <c r="S6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T6">
         <v>-1</v>
@@ -61586,16 +61586,16 @@
         <v>8</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="R7">
         <v>-1</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T7">
         <v>-1</v>
@@ -61607,7 +61607,7 @@
         <v>-1</v>
       </c>
       <c r="W7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X7">
         <v>7</v>
@@ -61675,16 +61675,16 @@
         <v>8</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R8">
         <v>-1</v>
       </c>
       <c r="S8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T8">
         <v>-1</v>
@@ -61699,7 +61699,7 @@
         <v>8</v>
       </c>
       <c r="X8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y8">
         <v>7</v>
@@ -61767,13 +61767,13 @@
         <v>6</v>
       </c>
       <c r="Q9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R9">
         <v>-1</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T9">
         <v>-1</v>
@@ -61794,7 +61794,7 @@
         <v>7</v>
       </c>
       <c r="Z9">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AA9">
         <v>7</v>
@@ -61853,16 +61853,16 @@
         <v>5</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="R10">
         <v>-1</v>
       </c>
       <c r="S10">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T10">
         <v>-1</v>
@@ -61877,13 +61877,13 @@
         <v>5</v>
       </c>
       <c r="X10">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Y10">
         <v>5</v>
       </c>
       <c r="Z10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AA10">
         <v>5</v>
@@ -61945,13 +61945,13 @@
         <v>10</v>
       </c>
       <c r="Q11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R11">
         <v>-1</v>
       </c>
       <c r="S11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T11">
         <v>-1</v>
@@ -62034,13 +62034,13 @@
         <v>8</v>
       </c>
       <c r="Q12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R12">
         <v>-1</v>
       </c>
       <c r="S12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T12">
         <v>-1</v>
@@ -62120,16 +62120,16 @@
         <v>6</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R13">
         <v>-1</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T13">
         <v>-1</v>
@@ -62209,16 +62209,16 @@
         <v>7</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="R14">
         <v>-1</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T14">
         <v>-1</v>
@@ -62298,16 +62298,16 @@
         <v>5</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R15">
         <v>-1</v>
       </c>
       <c r="S15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T15">
         <v>-1</v>
@@ -62319,7 +62319,7 @@
         <v>-1</v>
       </c>
       <c r="W15">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="X15">
         <v>7</v>
@@ -62328,7 +62328,7 @@
         <v>7</v>
       </c>
       <c r="Z15">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA15">
         <v>7</v>
@@ -62387,16 +62387,16 @@
         <v>8</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R16">
         <v>-1</v>
       </c>
       <c r="S16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T16">
         <v>-1</v>
@@ -62417,7 +62417,7 @@
         <v>8</v>
       </c>
       <c r="Z16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AA16">
         <v>8</v>
@@ -62479,13 +62479,13 @@
         <v>10</v>
       </c>
       <c r="Q17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="R17">
         <v>-1</v>
       </c>
       <c r="S17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T17">
         <v>-1</v>
@@ -62565,16 +62565,16 @@
         <v>5</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R18">
         <v>-1</v>
       </c>
       <c r="S18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T18">
         <v>-1</v>
@@ -62586,7 +62586,7 @@
         <v>-1</v>
       </c>
       <c r="W18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X18">
         <v>7</v>
@@ -62595,7 +62595,7 @@
         <v>7</v>
       </c>
       <c r="Z18">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA18">
         <v>7</v>
@@ -62657,13 +62657,13 @@
         <v>10</v>
       </c>
       <c r="Q19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="R19">
         <v>-1</v>
       </c>
       <c r="S19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T19">
         <v>-1</v>
@@ -62678,13 +62678,13 @@
         <v>8</v>
       </c>
       <c r="X19">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y19">
         <v>8</v>
       </c>
       <c r="Z19">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA19">
         <v>9</v>
@@ -62746,13 +62746,13 @@
         <v>9</v>
       </c>
       <c r="Q20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R20">
         <v>-1</v>
       </c>
       <c r="S20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T20">
         <v>-1</v>
@@ -62835,13 +62835,13 @@
         <v>8</v>
       </c>
       <c r="Q21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="R21">
         <v>-1</v>
       </c>
       <c r="S21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T21">
         <v>-1</v>
@@ -62862,7 +62862,7 @@
         <v>8</v>
       </c>
       <c r="Z21">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AA21">
         <v>9</v>
@@ -62921,16 +62921,16 @@
         <v>9</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q22">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R22">
         <v>-1</v>
       </c>
       <c r="S22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T22">
         <v>-1</v>
@@ -62942,7 +62942,7 @@
         <v>-1</v>
       </c>
       <c r="W22">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="X22">
         <v>7</v>
@@ -63010,16 +63010,16 @@
         <v>5</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="R23">
         <v>-1</v>
       </c>
       <c r="S23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T23">
         <v>-1</v>
@@ -63031,10 +63031,10 @@
         <v>-1</v>
       </c>
       <c r="W23">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X23">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Y23">
         <v>5</v>
@@ -63102,13 +63102,13 @@
         <v>7</v>
       </c>
       <c r="Q24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="R24">
         <v>-1</v>
       </c>
       <c r="S24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T24">
         <v>-1</v>
@@ -63123,7 +63123,7 @@
         <v>6</v>
       </c>
       <c r="X24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y24">
         <v>7</v>
@@ -63188,16 +63188,16 @@
         <v>8</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="R25">
         <v>-1</v>
       </c>
       <c r="S25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T25">
         <v>-1</v>
@@ -63209,7 +63209,7 @@
         <v>-1</v>
       </c>
       <c r="W25">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X25">
         <v>10</v>
@@ -63277,16 +63277,16 @@
         <v>5</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="R26">
         <v>-1</v>
       </c>
       <c r="S26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T26">
         <v>-1</v>
@@ -63301,13 +63301,13 @@
         <v>7</v>
       </c>
       <c r="X26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Y26">
         <v>7</v>
       </c>
       <c r="Z26">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA26">
         <v>7</v>
@@ -63369,13 +63369,13 @@
         <v>10</v>
       </c>
       <c r="Q27">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="R27">
         <v>-1</v>
       </c>
       <c r="S27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T27">
         <v>-1</v>
@@ -63390,7 +63390,7 @@
         <v>8</v>
       </c>
       <c r="X27">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y27">
         <v>7</v>
@@ -63458,13 +63458,13 @@
         <v>8</v>
       </c>
       <c r="Q28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R28">
         <v>-1</v>
       </c>
       <c r="S28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T28">
         <v>-1</v>
@@ -63547,13 +63547,13 @@
         <v>7</v>
       </c>
       <c r="Q29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="R29">
         <v>-1</v>
       </c>
       <c r="S29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T29">
         <v>-1</v>
@@ -63633,16 +63633,16 @@
         <v>7</v>
       </c>
       <c r="P30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="R30">
         <v>-1</v>
       </c>
       <c r="S30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T30">
         <v>-1</v>
@@ -63654,10 +63654,10 @@
         <v>-1</v>
       </c>
       <c r="W30">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X30">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Y30">
         <v>6</v>
@@ -63725,13 +63725,13 @@
         <v>9</v>
       </c>
       <c r="Q31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R31">
         <v>-1</v>
       </c>
       <c r="S31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T31">
         <v>-1</v>
@@ -63746,13 +63746,13 @@
         <v>9</v>
       </c>
       <c r="X31">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="Y31">
         <v>8</v>
       </c>
       <c r="Z31">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA31">
         <v>9</v>
@@ -67128,7 +67128,7 @@
         <v>5</v>
       </c>
       <c r="Q4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R4">
         <v>9</v>
@@ -67146,7 +67146,7 @@
         <v>5</v>
       </c>
       <c r="W4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X4">
         <v>6</v>
@@ -67205,7 +67205,7 @@
         <v>7</v>
       </c>
       <c r="Q5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R5">
         <v>10</v>
@@ -67223,7 +67223,7 @@
         <v>6</v>
       </c>
       <c r="W5">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X5">
         <v>10</v>
@@ -67282,7 +67282,7 @@
         <v>10</v>
       </c>
       <c r="Q6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="R6">
         <v>7</v>
@@ -67300,7 +67300,7 @@
         <v>9</v>
       </c>
       <c r="W6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X6">
         <v>8</v>
@@ -67359,7 +67359,7 @@
         <v>5</v>
       </c>
       <c r="Q7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="R7">
         <v>5</v>
@@ -67377,7 +67377,7 @@
         <v>5</v>
       </c>
       <c r="W7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="X7">
         <v>5</v>
@@ -67436,7 +67436,7 @@
         <v>9</v>
       </c>
       <c r="Q8">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R8">
         <v>10</v>
@@ -67454,7 +67454,7 @@
         <v>7</v>
       </c>
       <c r="W8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X8">
         <v>8</v>
@@ -67513,7 +67513,7 @@
         <v>9</v>
       </c>
       <c r="Q9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R9">
         <v>10</v>
@@ -67590,7 +67590,7 @@
         <v>5</v>
       </c>
       <c r="Q10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R10">
         <v>10</v>
@@ -67667,7 +67667,7 @@
         <v>5</v>
       </c>
       <c r="Q11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="R11">
         <v>5</v>
@@ -67685,7 +67685,7 @@
         <v>7</v>
       </c>
       <c r="W11">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X11">
         <v>8</v>
@@ -67744,7 +67744,7 @@
         <v>6</v>
       </c>
       <c r="Q12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R12">
         <v>7</v>
@@ -67762,7 +67762,7 @@
         <v>6</v>
       </c>
       <c r="W12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X12">
         <v>6</v>
@@ -67821,7 +67821,7 @@
         <v>6</v>
       </c>
       <c r="Q13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="R13">
         <v>8</v>
@@ -67839,7 +67839,7 @@
         <v>6</v>
       </c>
       <c r="W13">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X13">
         <v>9</v>
@@ -67898,7 +67898,7 @@
         <v>5</v>
       </c>
       <c r="Q14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R14">
         <v>5</v>
@@ -67916,7 +67916,7 @@
         <v>5</v>
       </c>
       <c r="W14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X14">
         <v>5</v>
@@ -67975,7 +67975,7 @@
         <v>9</v>
       </c>
       <c r="Q15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R15">
         <v>10</v>
@@ -68052,7 +68052,7 @@
         <v>8</v>
       </c>
       <c r="Q16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="R16">
         <v>5</v>
@@ -68129,7 +68129,7 @@
         <v>5</v>
       </c>
       <c r="Q17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="R17">
         <v>10</v>
@@ -68206,7 +68206,7 @@
         <v>8</v>
       </c>
       <c r="Q18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R18">
         <v>10</v>
@@ -68283,7 +68283,7 @@
         <v>7</v>
       </c>
       <c r="Q19">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R19">
         <v>10</v>
@@ -68301,7 +68301,7 @@
         <v>6</v>
       </c>
       <c r="W19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X19">
         <v>9</v>
@@ -68360,7 +68360,7 @@
         <v>9</v>
       </c>
       <c r="Q20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R20">
         <v>10</v>
@@ -68437,7 +68437,7 @@
         <v>7</v>
       </c>
       <c r="Q21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R21">
         <v>10</v>
@@ -68514,7 +68514,7 @@
         <v>10</v>
       </c>
       <c r="Q22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R22">
         <v>7</v>
@@ -68591,7 +68591,7 @@
         <v>8</v>
       </c>
       <c r="Q23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R23">
         <v>10</v>
@@ -68668,7 +68668,7 @@
         <v>7</v>
       </c>
       <c r="Q24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R24">
         <v>6</v>
@@ -68686,7 +68686,7 @@
         <v>6</v>
       </c>
       <c r="W24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X24">
         <v>6</v>
@@ -68745,7 +68745,7 @@
         <v>8</v>
       </c>
       <c r="Q25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R25">
         <v>10</v>
@@ -68822,7 +68822,7 @@
         <v>8</v>
       </c>
       <c r="Q26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R26">
         <v>10</v>
@@ -68899,7 +68899,7 @@
         <v>10</v>
       </c>
       <c r="Q27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R27">
         <v>10</v>
@@ -68917,7 +68917,7 @@
         <v>10</v>
       </c>
       <c r="W27">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="X27">
         <v>10</v>
@@ -68976,7 +68976,7 @@
         <v>7</v>
       </c>
       <c r="Q28">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R28">
         <v>7</v>
@@ -69053,7 +69053,7 @@
         <v>7</v>
       </c>
       <c r="Q29">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R29">
         <v>9</v>
@@ -69130,7 +69130,7 @@
         <v>8</v>
       </c>
       <c r="Q30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R30">
         <v>10</v>
@@ -69148,7 +69148,7 @@
         <v>6</v>
       </c>
       <c r="W30">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X30">
         <v>9</v>
@@ -69207,7 +69207,7 @@
         <v>8</v>
       </c>
       <c r="Q31">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R31">
         <v>10</v>
@@ -69225,7 +69225,7 @@
         <v>8</v>
       </c>
       <c r="W31">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="X31">
         <v>10</v>
@@ -69284,7 +69284,7 @@
         <v>7</v>
       </c>
       <c r="Q32">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R32">
         <v>7</v>
@@ -69302,7 +69302,7 @@
         <v>6</v>
       </c>
       <c r="W32">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X32">
         <v>6</v>
@@ -69361,7 +69361,7 @@
         <v>7</v>
       </c>
       <c r="Q33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R33">
         <v>8</v>
@@ -69438,7 +69438,7 @@
         <v>7</v>
       </c>
       <c r="Q34">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="R34">
         <v>8</v>
@@ -69515,7 +69515,7 @@
         <v>7</v>
       </c>
       <c r="Q35">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="R35">
         <v>5</v>
@@ -69533,7 +69533,7 @@
         <v>6</v>
       </c>
       <c r="W35">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X35">
         <v>5</v>
@@ -69592,7 +69592,7 @@
         <v>7</v>
       </c>
       <c r="Q36">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R36">
         <v>10</v>
@@ -71199,7 +71199,7 @@
         <v>8</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q4">
         <v>8</v>
@@ -71276,7 +71276,7 @@
         <v>7</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q5">
         <v>9</v>
@@ -71353,7 +71353,7 @@
         <v>7</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q6">
         <v>9</v>
@@ -71430,7 +71430,7 @@
         <v>10</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q7">
         <v>9</v>
@@ -71507,7 +71507,7 @@
         <v>5</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="Q8">
         <v>9</v>
@@ -71584,7 +71584,7 @@
         <v>7</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q9">
         <v>8</v>
@@ -71602,7 +71602,7 @@
         <v>7</v>
       </c>
       <c r="V9">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W9">
         <v>8</v>
@@ -71661,7 +71661,7 @@
         <v>10</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q10">
         <v>8</v>
@@ -71679,7 +71679,7 @@
         <v>9</v>
       </c>
       <c r="V10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W10">
         <v>8</v>
@@ -71738,7 +71738,7 @@
         <v>9</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q11">
         <v>9</v>
@@ -71815,7 +71815,7 @@
         <v>5</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q12">
         <v>8</v>
@@ -71892,7 +71892,7 @@
         <v>9</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q13">
         <v>8</v>
@@ -71969,7 +71969,7 @@
         <v>10</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q14">
         <v>10</v>
@@ -72046,7 +72046,7 @@
         <v>8</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q15">
         <v>9</v>
@@ -72123,7 +72123,7 @@
         <v>8</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q16">
         <v>9</v>
@@ -72141,7 +72141,7 @@
         <v>7</v>
       </c>
       <c r="V16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W16">
         <v>8</v>
@@ -72200,7 +72200,7 @@
         <v>10</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q17">
         <v>8</v>
@@ -72277,7 +72277,7 @@
         <v>6</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q18">
         <v>9</v>
@@ -72295,7 +72295,7 @@
         <v>7</v>
       </c>
       <c r="V18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W18">
         <v>8</v>
@@ -72354,7 +72354,7 @@
         <v>7</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q19">
         <v>9</v>
@@ -72431,7 +72431,7 @@
         <v>7</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q20">
         <v>9</v>
@@ -72449,7 +72449,7 @@
         <v>8</v>
       </c>
       <c r="V20">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W20">
         <v>8</v>
@@ -72508,7 +72508,7 @@
         <v>10</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q21">
         <v>9</v>
@@ -72585,7 +72585,7 @@
         <v>9</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q22">
         <v>9</v>
@@ -72662,7 +72662,7 @@
         <v>10</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q23">
         <v>9</v>
@@ -72739,7 +72739,7 @@
         <v>7</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q24">
         <v>9</v>
@@ -72757,7 +72757,7 @@
         <v>6</v>
       </c>
       <c r="V24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W24">
         <v>8</v>
@@ -72816,7 +72816,7 @@
         <v>8</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q25">
         <v>9</v>
@@ -72893,7 +72893,7 @@
         <v>7</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q26">
         <v>9</v>
@@ -72970,7 +72970,7 @@
         <v>9</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q27">
         <v>9</v>
@@ -72988,7 +72988,7 @@
         <v>7</v>
       </c>
       <c r="V27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W27">
         <v>8</v>
@@ -73047,7 +73047,7 @@
         <v>6</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q28">
         <v>9</v>
@@ -73065,7 +73065,7 @@
         <v>7</v>
       </c>
       <c r="V28">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W28">
         <v>8</v>
@@ -73124,7 +73124,7 @@
         <v>8</v>
       </c>
       <c r="P29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q29">
         <v>9</v>
@@ -73142,7 +73142,7 @@
         <v>7</v>
       </c>
       <c r="V29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W29">
         <v>8</v>
@@ -73343,7 +73343,7 @@
         <v>10</v>
       </c>
       <c r="R4">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S4">
         <v>8</v>
@@ -73361,7 +73361,7 @@
         <v>8</v>
       </c>
       <c r="X4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y4">
         <v>6</v>
@@ -73420,7 +73420,7 @@
         <v>10</v>
       </c>
       <c r="R5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S5">
         <v>10</v>
@@ -73497,7 +73497,7 @@
         <v>10</v>
       </c>
       <c r="R6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S6">
         <v>8</v>
@@ -73538,7 +73538,7 @@
         <v>6</v>
       </c>
       <c r="F7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="G7">
         <v>6</v>
@@ -73556,7 +73556,7 @@
         <v>6</v>
       </c>
       <c r="L7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="M7">
         <v>6</v>
@@ -73574,7 +73574,7 @@
         <v>6</v>
       </c>
       <c r="R7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="S7">
         <v>8</v>
@@ -73592,7 +73592,7 @@
         <v>6</v>
       </c>
       <c r="X7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Y7">
         <v>7</v>
@@ -73651,7 +73651,7 @@
         <v>10</v>
       </c>
       <c r="R8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S8">
         <v>10</v>
@@ -73728,7 +73728,7 @@
         <v>10</v>
       </c>
       <c r="R9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S9">
         <v>5</v>
@@ -73746,7 +73746,7 @@
         <v>10</v>
       </c>
       <c r="X9">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y9">
         <v>6</v>
@@ -73805,7 +73805,7 @@
         <v>10</v>
       </c>
       <c r="R10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S10">
         <v>10</v>
@@ -73882,7 +73882,7 @@
         <v>10</v>
       </c>
       <c r="R11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S11">
         <v>10</v>
@@ -73959,7 +73959,7 @@
         <v>10</v>
       </c>
       <c r="R12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S12">
         <v>9</v>
@@ -74036,7 +74036,7 @@
         <v>10</v>
       </c>
       <c r="R13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S13">
         <v>7</v>
@@ -74113,7 +74113,7 @@
         <v>10</v>
       </c>
       <c r="R14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S14">
         <v>8</v>
@@ -74190,7 +74190,7 @@
         <v>10</v>
       </c>
       <c r="R15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S15">
         <v>5</v>
@@ -74267,7 +74267,7 @@
         <v>10</v>
       </c>
       <c r="R16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S16">
         <v>10</v>

</xml_diff>

<commit_message>
Estadisticos Tercer Parcial 8 Tarde
</commit_message>
<xml_diff>
--- a/Calificaciones20231.xlsx
+++ b/Calificaciones20231.xlsx
@@ -22850,7 +22850,7 @@
         <v>6</v>
       </c>
       <c r="N23">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="O23">
         <v>7</v>
@@ -22868,7 +22868,7 @@
         <v>7</v>
       </c>
       <c r="T23">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="U23">
         <v>5</v>
@@ -23934,7 +23934,7 @@
         <v>8</v>
       </c>
       <c r="V10">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="W10">
         <v>9</v>
@@ -29559,7 +29559,7 @@
         <v>9</v>
       </c>
       <c r="O17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P17">
         <v>6</v>
@@ -29577,7 +29577,7 @@
         <v>9</v>
       </c>
       <c r="U17">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="V17">
         <v>7</v>
@@ -30868,7 +30868,7 @@
         <v>5</v>
       </c>
       <c r="O34">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="P34">
         <v>10</v>
@@ -30886,7 +30886,7 @@
         <v>7</v>
       </c>
       <c r="U34">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="V34">
         <v>7</v>
@@ -31253,7 +31253,7 @@
         <v>10</v>
       </c>
       <c r="O39">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="P39">
         <v>6</v>
@@ -31503,7 +31503,7 @@
         <v>0</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W4">
         <v>5</v>
@@ -31592,7 +31592,7 @@
         <v>0</v>
       </c>
       <c r="V5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W5">
         <v>5</v>
@@ -31681,7 +31681,7 @@
         <v>8</v>
       </c>
       <c r="V6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W6">
         <v>7</v>
@@ -31770,7 +31770,7 @@
         <v>10</v>
       </c>
       <c r="V7">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W7">
         <v>6</v>
@@ -31859,7 +31859,7 @@
         <v>5</v>
       </c>
       <c r="V8">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W8">
         <v>6</v>
@@ -31948,7 +31948,7 @@
         <v>0</v>
       </c>
       <c r="V9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W9">
         <v>5</v>
@@ -32037,7 +32037,7 @@
         <v>10</v>
       </c>
       <c r="V10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W10">
         <v>8</v>
@@ -32126,7 +32126,7 @@
         <v>7</v>
       </c>
       <c r="V11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W11">
         <v>5</v>
@@ -32215,7 +32215,7 @@
         <v>8</v>
       </c>
       <c r="V12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W12">
         <v>5</v>
@@ -32236,7 +32236,7 @@
         <v>6</v>
       </c>
       <c r="AC12">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:29">
@@ -32304,7 +32304,7 @@
         <v>5</v>
       </c>
       <c r="V13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W13">
         <v>5</v>
@@ -32393,7 +32393,7 @@
         <v>10</v>
       </c>
       <c r="V14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W14">
         <v>7</v>
@@ -32414,7 +32414,7 @@
         <v>10</v>
       </c>
       <c r="AC14">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:29">
@@ -32482,7 +32482,7 @@
         <v>0</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W15">
         <v>5</v>
@@ -32571,7 +32571,7 @@
         <v>8</v>
       </c>
       <c r="V16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W16">
         <v>5</v>
@@ -32660,7 +32660,7 @@
         <v>8</v>
       </c>
       <c r="V17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W17">
         <v>5</v>
@@ -32749,7 +32749,7 @@
         <v>8</v>
       </c>
       <c r="V18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W18">
         <v>5</v>
@@ -32838,7 +32838,7 @@
         <v>8</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W19">
         <v>5</v>
@@ -32927,7 +32927,7 @@
         <v>10</v>
       </c>
       <c r="V20">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W20">
         <v>6</v>
@@ -32948,7 +32948,7 @@
         <v>9</v>
       </c>
       <c r="AC20">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:29">
@@ -33016,7 +33016,7 @@
         <v>5</v>
       </c>
       <c r="V21">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W21">
         <v>5</v>
@@ -33105,7 +33105,7 @@
         <v>5</v>
       </c>
       <c r="V22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W22">
         <v>5</v>
@@ -33194,7 +33194,7 @@
         <v>7</v>
       </c>
       <c r="V23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W23">
         <v>5</v>
@@ -33283,7 +33283,7 @@
         <v>0</v>
       </c>
       <c r="V24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W24">
         <v>5</v>
@@ -33372,7 +33372,7 @@
         <v>5</v>
       </c>
       <c r="V25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W25">
         <v>5</v>
@@ -33461,7 +33461,7 @@
         <v>10</v>
       </c>
       <c r="V26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W26">
         <v>6</v>
@@ -33482,7 +33482,7 @@
         <v>9</v>
       </c>
       <c r="AC26">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" spans="1:29">
@@ -33550,7 +33550,7 @@
         <v>8</v>
       </c>
       <c r="V27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W27">
         <v>5</v>
@@ -33571,7 +33571,7 @@
         <v>6</v>
       </c>
       <c r="AC27">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:29">
@@ -33639,7 +33639,7 @@
         <v>10</v>
       </c>
       <c r="V28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W28">
         <v>7</v>
@@ -33728,7 +33728,7 @@
         <v>0</v>
       </c>
       <c r="V29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W29">
         <v>5</v>
@@ -33817,7 +33817,7 @@
         <v>10</v>
       </c>
       <c r="V30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W30">
         <v>7</v>
@@ -33906,7 +33906,7 @@
         <v>7</v>
       </c>
       <c r="V31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W31">
         <v>5</v>
@@ -33995,7 +33995,7 @@
         <v>10</v>
       </c>
       <c r="V32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W32">
         <v>6</v>
@@ -34084,7 +34084,7 @@
         <v>10</v>
       </c>
       <c r="V33">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W33">
         <v>5</v>
@@ -34173,7 +34173,7 @@
         <v>5</v>
       </c>
       <c r="V34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W34">
         <v>5</v>
@@ -34262,7 +34262,7 @@
         <v>10</v>
       </c>
       <c r="V35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W35">
         <v>7</v>
@@ -34283,7 +34283,7 @@
         <v>10</v>
       </c>
       <c r="AC35">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:29">
@@ -34351,7 +34351,7 @@
         <v>7</v>
       </c>
       <c r="V36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W36">
         <v>5</v>
@@ -34440,7 +34440,7 @@
         <v>10</v>
       </c>
       <c r="V37">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W37">
         <v>8</v>
@@ -34529,7 +34529,7 @@
         <v>7</v>
       </c>
       <c r="V38">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W38">
         <v>5</v>
@@ -34550,7 +34550,7 @@
         <v>6</v>
       </c>
       <c r="AC38">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:29">
@@ -34618,7 +34618,7 @@
         <v>10</v>
       </c>
       <c r="V39">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W39">
         <v>5</v>
@@ -40752,7 +40752,7 @@
         <v>5</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q4">
         <v>5</v>
@@ -40770,7 +40770,7 @@
         <v>6</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W4">
         <v>5</v>
@@ -40859,7 +40859,7 @@
         <v>8</v>
       </c>
       <c r="V5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W5">
         <v>7</v>
@@ -40948,7 +40948,7 @@
         <v>5</v>
       </c>
       <c r="V6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W6">
         <v>5</v>
@@ -41037,7 +41037,7 @@
         <v>6</v>
       </c>
       <c r="V7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W7">
         <v>6</v>
@@ -41126,7 +41126,7 @@
         <v>6</v>
       </c>
       <c r="V8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W8">
         <v>7</v>
@@ -41147,7 +41147,7 @@
         <v>7</v>
       </c>
       <c r="AC8">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:29">
@@ -41215,7 +41215,7 @@
         <v>8</v>
       </c>
       <c r="V9">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W9">
         <v>7</v>
@@ -41304,7 +41304,7 @@
         <v>8</v>
       </c>
       <c r="V10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W10">
         <v>7</v>
@@ -41325,7 +41325,7 @@
         <v>8</v>
       </c>
       <c r="AC10">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:29">
@@ -41393,7 +41393,7 @@
         <v>5</v>
       </c>
       <c r="V11">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W11">
         <v>7</v>
@@ -41482,7 +41482,7 @@
         <v>6</v>
       </c>
       <c r="V12">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W12">
         <v>8</v>
@@ -41571,7 +41571,7 @@
         <v>6</v>
       </c>
       <c r="V13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W13">
         <v>6</v>
@@ -41660,7 +41660,7 @@
         <v>7</v>
       </c>
       <c r="V14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W14">
         <v>6</v>
@@ -41749,7 +41749,7 @@
         <v>9</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W15">
         <v>8</v>
@@ -41770,7 +41770,7 @@
         <v>8</v>
       </c>
       <c r="AC15">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:29">
@@ -41838,7 +41838,7 @@
         <v>5</v>
       </c>
       <c r="V16">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W16">
         <v>7</v>
@@ -41927,7 +41927,7 @@
         <v>9</v>
       </c>
       <c r="V17">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W17">
         <v>8</v>
@@ -42016,7 +42016,7 @@
         <v>6</v>
       </c>
       <c r="V18">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W18">
         <v>6</v>
@@ -42105,7 +42105,7 @@
         <v>8</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W19">
         <v>6</v>
@@ -42126,7 +42126,7 @@
         <v>7</v>
       </c>
       <c r="AC19">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:29">
@@ -42194,7 +42194,7 @@
         <v>5</v>
       </c>
       <c r="V20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W20">
         <v>5</v>
@@ -42283,7 +42283,7 @@
         <v>6</v>
       </c>
       <c r="V21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W21">
         <v>6</v>
@@ -42304,7 +42304,7 @@
         <v>6</v>
       </c>
       <c r="AC21">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:29">
@@ -42354,7 +42354,7 @@
         <v>5</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q22">
         <v>7</v>
@@ -42372,10 +42372,10 @@
         <v>5</v>
       </c>
       <c r="V22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W22">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="X22">
         <v>6</v>
@@ -42461,7 +42461,7 @@
         <v>6</v>
       </c>
       <c r="V23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W23">
         <v>6</v>
@@ -42550,7 +42550,7 @@
         <v>8</v>
       </c>
       <c r="V24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W24">
         <v>8</v>
@@ -42639,7 +42639,7 @@
         <v>6</v>
       </c>
       <c r="V25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W25">
         <v>8</v>
@@ -42728,7 +42728,7 @@
         <v>7</v>
       </c>
       <c r="V26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W26">
         <v>6</v>
@@ -42749,7 +42749,7 @@
         <v>6</v>
       </c>
       <c r="AC26">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:29">
@@ -42817,7 +42817,7 @@
         <v>6</v>
       </c>
       <c r="V27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W27">
         <v>6</v>
@@ -42888,7 +42888,7 @@
         <v>6</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q28">
         <v>8</v>
@@ -42906,10 +42906,10 @@
         <v>7</v>
       </c>
       <c r="V28">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W28">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="X28">
         <v>7</v>
@@ -42995,7 +42995,7 @@
         <v>6</v>
       </c>
       <c r="V29">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W29">
         <v>7</v>
@@ -43084,7 +43084,7 @@
         <v>8</v>
       </c>
       <c r="V30">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W30">
         <v>7</v>
@@ -43105,7 +43105,7 @@
         <v>6</v>
       </c>
       <c r="AC30">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:29">
@@ -43173,7 +43173,7 @@
         <v>7</v>
       </c>
       <c r="V31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W31">
         <v>7</v>
@@ -43194,7 +43194,7 @@
         <v>7</v>
       </c>
       <c r="AC31">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:29">
@@ -43262,7 +43262,7 @@
         <v>5</v>
       </c>
       <c r="V32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W32">
         <v>5</v>
@@ -43351,7 +43351,7 @@
         <v>8</v>
       </c>
       <c r="V33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W33">
         <v>7</v>
@@ -43440,7 +43440,7 @@
         <v>5</v>
       </c>
       <c r="V34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W34">
         <v>6</v>
@@ -43529,7 +43529,7 @@
         <v>9</v>
       </c>
       <c r="V35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W35">
         <v>10</v>
@@ -43618,7 +43618,7 @@
         <v>5</v>
       </c>
       <c r="V36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W36">
         <v>5</v>
@@ -43707,7 +43707,7 @@
         <v>7</v>
       </c>
       <c r="V37">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W37">
         <v>7</v>
@@ -43778,7 +43778,7 @@
         <v>5</v>
       </c>
       <c r="P38">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q38">
         <v>8</v>
@@ -43796,10 +43796,10 @@
         <v>5</v>
       </c>
       <c r="V38">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W38">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X38">
         <v>6</v>
@@ -43885,7 +43885,7 @@
         <v>7</v>
       </c>
       <c r="V39">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W39">
         <v>7</v>
@@ -43974,7 +43974,7 @@
         <v>7</v>
       </c>
       <c r="V40">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W40">
         <v>7</v>
@@ -44063,7 +44063,7 @@
         <v>9</v>
       </c>
       <c r="V41">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W41">
         <v>9</v>
@@ -44152,7 +44152,7 @@
         <v>5</v>
       </c>
       <c r="V42">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W42">
         <v>5</v>
@@ -50017,7 +50017,7 @@
         <v>7</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T9">
         <v>6</v>
@@ -50402,7 +50402,7 @@
         <v>8</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T14">
         <v>7</v>
@@ -51278,7 +51278,7 @@
         <v>10</v>
       </c>
       <c r="S26">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T26">
         <v>7</v>
@@ -51296,7 +51296,7 @@
         <v>8</v>
       </c>
       <c r="Y26">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="27" spans="1:25">
@@ -52027,7 +52027,7 @@
         <v>7</v>
       </c>
       <c r="R9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S9">
         <v>5</v>
@@ -52181,7 +52181,7 @@
         <v>5</v>
       </c>
       <c r="R11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S11">
         <v>5</v>
@@ -52489,7 +52489,7 @@
         <v>5</v>
       </c>
       <c r="R15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S15">
         <v>5</v>
@@ -53182,7 +53182,7 @@
         <v>8</v>
       </c>
       <c r="R24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S24">
         <v>8</v>
@@ -53203,7 +53203,7 @@
         <v>5</v>
       </c>
       <c r="Y24">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:25">
@@ -53596,7 +53596,7 @@
         <v>5</v>
       </c>
       <c r="R30">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S30">
         <v>5</v>
@@ -53933,7 +53933,7 @@
         <v>7</v>
       </c>
       <c r="R35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="S35">
         <v>5</v>
@@ -54125,7 +54125,7 @@
         <v>8</v>
       </c>
       <c r="U38">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V38">
         <v>8</v>
@@ -57090,7 +57090,7 @@
         <v>0</v>
       </c>
       <c r="Q9">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="R9">
         <v>0</v>
@@ -57205,7 +57205,7 @@
         <v>10</v>
       </c>
       <c r="D11">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E11">
         <v>7</v>
@@ -57259,7 +57259,7 @@
         <v>10</v>
       </c>
       <c r="V11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="W11">
         <v>9</v>
@@ -57350,7 +57350,7 @@
         <v>5</v>
       </c>
       <c r="Q13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="R13">
         <v>7</v>
@@ -57368,7 +57368,7 @@
         <v>5</v>
       </c>
       <c r="W13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X13">
         <v>6</v>
@@ -60687,7 +60687,7 @@
         <v>10</v>
       </c>
       <c r="J28">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K28">
         <v>9</v>
@@ -60723,7 +60723,7 @@
         <v>10</v>
       </c>
       <c r="V28">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="W28">
         <v>9</v>
@@ -61325,19 +61325,19 @@
         <v>7</v>
       </c>
       <c r="R4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S4">
         <v>8</v>
       </c>
       <c r="T4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="U4">
         <v>6</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W4">
         <v>7</v>
@@ -61414,19 +61414,19 @@
         <v>7</v>
       </c>
       <c r="R5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="S5">
         <v>6</v>
       </c>
       <c r="T5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="U5">
         <v>6</v>
       </c>
       <c r="V5">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W5">
         <v>8</v>
@@ -61503,19 +61503,19 @@
         <v>9</v>
       </c>
       <c r="R6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S6">
         <v>6</v>
       </c>
       <c r="T6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U6">
         <v>6</v>
       </c>
       <c r="V6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W6">
         <v>8</v>
@@ -61524,19 +61524,19 @@
         <v>8</v>
       </c>
       <c r="Y6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Z6">
         <v>7</v>
       </c>
       <c r="AA6">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AB6">
         <v>8</v>
       </c>
       <c r="AC6">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:29">
@@ -61592,19 +61592,19 @@
         <v>6</v>
       </c>
       <c r="R7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S7">
         <v>6</v>
       </c>
       <c r="T7">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U7">
         <v>6</v>
       </c>
       <c r="V7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W7">
         <v>5</v>
@@ -61613,13 +61613,13 @@
         <v>7</v>
       </c>
       <c r="Y7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Z7">
         <v>6</v>
       </c>
       <c r="AA7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AB7">
         <v>6</v>
@@ -61681,19 +61681,19 @@
         <v>8</v>
       </c>
       <c r="R8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S8">
         <v>8</v>
       </c>
       <c r="T8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U8">
         <v>7</v>
       </c>
       <c r="V8">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W8">
         <v>8</v>
@@ -61702,7 +61702,7 @@
         <v>6</v>
       </c>
       <c r="Y8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Z8">
         <v>7</v>
@@ -61770,19 +61770,19 @@
         <v>7</v>
       </c>
       <c r="R9">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S9">
         <v>6</v>
       </c>
       <c r="T9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U9">
         <v>6</v>
       </c>
       <c r="V9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W9">
         <v>6</v>
@@ -61797,7 +61797,7 @@
         <v>6</v>
       </c>
       <c r="AA9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AB9">
         <v>8</v>
@@ -61859,19 +61859,19 @@
         <v>5</v>
       </c>
       <c r="R10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S10">
         <v>0</v>
       </c>
       <c r="T10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="U10">
         <v>5</v>
       </c>
       <c r="V10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W10">
         <v>5</v>
@@ -61948,19 +61948,19 @@
         <v>8</v>
       </c>
       <c r="R11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S11">
         <v>7</v>
       </c>
       <c r="T11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U11">
         <v>8</v>
       </c>
       <c r="V11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W11">
         <v>8</v>
@@ -62037,19 +62037,19 @@
         <v>8</v>
       </c>
       <c r="R12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S12">
         <v>6</v>
       </c>
       <c r="T12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U12">
         <v>6</v>
       </c>
       <c r="V12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W12">
         <v>7</v>
@@ -62058,7 +62058,7 @@
         <v>7</v>
       </c>
       <c r="Y12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Z12">
         <v>6</v>
@@ -62070,7 +62070,7 @@
         <v>6</v>
       </c>
       <c r="AC12">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:29">
@@ -62126,19 +62126,19 @@
         <v>8</v>
       </c>
       <c r="R13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S13">
         <v>7</v>
       </c>
       <c r="T13">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="U13">
         <v>6</v>
       </c>
       <c r="V13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W13">
         <v>5</v>
@@ -62147,19 +62147,19 @@
         <v>7</v>
       </c>
       <c r="Y13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Z13">
         <v>6</v>
       </c>
       <c r="AA13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AB13">
         <v>6</v>
       </c>
       <c r="AC13">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:29">
@@ -62215,19 +62215,19 @@
         <v>9</v>
       </c>
       <c r="R14">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S14">
         <v>8</v>
       </c>
       <c r="T14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U14">
         <v>7</v>
       </c>
       <c r="V14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W14">
         <v>9</v>
@@ -62242,13 +62242,13 @@
         <v>8</v>
       </c>
       <c r="AA14">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AB14">
         <v>9</v>
       </c>
       <c r="AC14">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:29">
@@ -62304,19 +62304,19 @@
         <v>8</v>
       </c>
       <c r="R15">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S15">
         <v>6</v>
       </c>
       <c r="T15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U15">
         <v>8</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W15">
         <v>7</v>
@@ -62331,13 +62331,13 @@
         <v>7</v>
       </c>
       <c r="AA15">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AB15">
         <v>7</v>
       </c>
       <c r="AC15">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:29">
@@ -62393,19 +62393,19 @@
         <v>8</v>
       </c>
       <c r="R16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S16">
         <v>5</v>
       </c>
       <c r="T16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U16">
         <v>7</v>
       </c>
       <c r="V16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W16">
         <v>7</v>
@@ -62420,7 +62420,7 @@
         <v>6</v>
       </c>
       <c r="AA16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AB16">
         <v>8</v>
@@ -62482,19 +62482,19 @@
         <v>10</v>
       </c>
       <c r="R17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S17">
         <v>10</v>
       </c>
       <c r="T17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U17">
         <v>10</v>
       </c>
       <c r="V17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W17">
         <v>9</v>
@@ -62509,13 +62509,13 @@
         <v>9</v>
       </c>
       <c r="AA17">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AB17">
         <v>10</v>
       </c>
       <c r="AC17">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:29">
@@ -62571,19 +62571,19 @@
         <v>8</v>
       </c>
       <c r="R18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S18">
         <v>6</v>
       </c>
       <c r="T18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U18">
         <v>7</v>
       </c>
       <c r="V18">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W18">
         <v>6</v>
@@ -62598,13 +62598,13 @@
         <v>7</v>
       </c>
       <c r="AA18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AB18">
         <v>7</v>
       </c>
       <c r="AC18">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19" spans="1:29">
@@ -62660,19 +62660,19 @@
         <v>9</v>
       </c>
       <c r="R19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S19">
         <v>7</v>
       </c>
       <c r="T19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U19">
         <v>9</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W19">
         <v>8</v>
@@ -62749,19 +62749,19 @@
         <v>8</v>
       </c>
       <c r="R20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S20">
         <v>8</v>
       </c>
       <c r="T20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U20">
         <v>7</v>
       </c>
       <c r="V20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W20">
         <v>7</v>
@@ -62782,7 +62782,7 @@
         <v>7</v>
       </c>
       <c r="AC20">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" spans="1:29">
@@ -62838,19 +62838,19 @@
         <v>9</v>
       </c>
       <c r="R21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S21">
         <v>5</v>
       </c>
       <c r="T21">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U21">
         <v>7</v>
       </c>
       <c r="V21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W21">
         <v>7</v>
@@ -62927,19 +62927,19 @@
         <v>7</v>
       </c>
       <c r="R22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="S22">
         <v>6</v>
       </c>
       <c r="T22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="U22">
         <v>7</v>
       </c>
       <c r="V22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W22">
         <v>5</v>
@@ -63016,19 +63016,19 @@
         <v>6</v>
       </c>
       <c r="R23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="S23">
         <v>6</v>
       </c>
       <c r="T23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="U23">
         <v>6</v>
       </c>
       <c r="V23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W23">
         <v>5</v>
@@ -63043,13 +63043,13 @@
         <v>6</v>
       </c>
       <c r="AA23">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AB23">
         <v>7</v>
       </c>
       <c r="AC23">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:29">
@@ -63105,19 +63105,19 @@
         <v>10</v>
       </c>
       <c r="R24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S24">
         <v>7</v>
       </c>
       <c r="T24">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U24">
         <v>8</v>
       </c>
       <c r="V24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W24">
         <v>6</v>
@@ -63194,19 +63194,19 @@
         <v>10</v>
       </c>
       <c r="R25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S25">
         <v>8</v>
       </c>
       <c r="T25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="U25">
         <v>7</v>
       </c>
       <c r="V25">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W25">
         <v>9</v>
@@ -63283,19 +63283,19 @@
         <v>5</v>
       </c>
       <c r="R26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S26">
         <v>6</v>
       </c>
       <c r="T26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="U26">
         <v>6</v>
       </c>
       <c r="V26">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W26">
         <v>7</v>
@@ -63316,7 +63316,7 @@
         <v>7</v>
       </c>
       <c r="AC26">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:29">
@@ -63372,19 +63372,19 @@
         <v>9</v>
       </c>
       <c r="R27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S27">
         <v>6</v>
       </c>
       <c r="T27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="U27">
         <v>6</v>
       </c>
       <c r="V27">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W27">
         <v>8</v>
@@ -63399,13 +63399,13 @@
         <v>7</v>
       </c>
       <c r="AA27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AB27">
         <v>8</v>
       </c>
       <c r="AC27">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:29">
@@ -63461,19 +63461,19 @@
         <v>8</v>
       </c>
       <c r="R28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S28">
         <v>6</v>
       </c>
       <c r="T28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="U28">
         <v>7</v>
       </c>
       <c r="V28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W28">
         <v>6</v>
@@ -63550,19 +63550,19 @@
         <v>9</v>
       </c>
       <c r="R29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S29">
         <v>9</v>
       </c>
       <c r="T29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="U29">
         <v>6</v>
       </c>
       <c r="V29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W29">
         <v>7</v>
@@ -63571,7 +63571,7 @@
         <v>9</v>
       </c>
       <c r="Y29">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Z29">
         <v>8</v>
@@ -63639,19 +63639,19 @@
         <v>6</v>
       </c>
       <c r="R30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S30">
         <v>6</v>
       </c>
       <c r="T30">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="U30">
         <v>6</v>
       </c>
       <c r="V30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="W30">
         <v>6</v>
@@ -63660,7 +63660,7 @@
         <v>6</v>
       </c>
       <c r="Y30">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Z30">
         <v>6</v>
@@ -63728,19 +63728,19 @@
         <v>8</v>
       </c>
       <c r="R31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S31">
         <v>7</v>
       </c>
       <c r="T31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="U31">
         <v>7</v>
       </c>
       <c r="V31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="W31">
         <v>9</v>
@@ -70664,7 +70664,7 @@
         <v>6</v>
       </c>
       <c r="U15">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="V15">
         <v>6</v>
@@ -80371,7 +80371,7 @@
         <v>8</v>
       </c>
       <c r="AA28">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AB28">
         <v>9</v>

</xml_diff>

<commit_message>
Estadisticos Tercer Parcial 8 Noche
</commit_message>
<xml_diff>
--- a/Calificaciones20231.xlsx
+++ b/Calificaciones20231.xlsx
@@ -34841,7 +34841,7 @@
         <v>5</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q4">
         <v>5</v>
@@ -34930,7 +34930,7 @@
         <v>5</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q5">
         <v>6</v>
@@ -34951,7 +34951,7 @@
         <v>9</v>
       </c>
       <c r="W5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X5">
         <v>6</v>
@@ -35019,7 +35019,7 @@
         <v>10</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q6">
         <v>9</v>
@@ -35108,7 +35108,7 @@
         <v>8</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q7">
         <v>8</v>
@@ -35197,7 +35197,7 @@
         <v>5</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q8">
         <v>5</v>
@@ -35286,7 +35286,7 @@
         <v>10</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q9">
         <v>8</v>
@@ -35375,7 +35375,7 @@
         <v>7</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q10">
         <v>8</v>
@@ -35464,7 +35464,7 @@
         <v>7</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q11">
         <v>8</v>
@@ -35553,7 +35553,7 @@
         <v>10</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q12">
         <v>7</v>
@@ -35642,7 +35642,7 @@
         <v>7</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q13">
         <v>7</v>
@@ -35731,7 +35731,7 @@
         <v>5</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q14">
         <v>5</v>
@@ -35820,7 +35820,7 @@
         <v>5</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q15">
         <v>5</v>
@@ -35841,7 +35841,7 @@
         <v>8</v>
       </c>
       <c r="W15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X15">
         <v>5</v>
@@ -35909,7 +35909,7 @@
         <v>8</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q16">
         <v>6</v>
@@ -35998,7 +35998,7 @@
         <v>5</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q17">
         <v>5</v>
@@ -36019,7 +36019,7 @@
         <v>5</v>
       </c>
       <c r="W17">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X17">
         <v>5</v>
@@ -36087,7 +36087,7 @@
         <v>7</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q18">
         <v>7</v>
@@ -36176,7 +36176,7 @@
         <v>9</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q19">
         <v>8</v>
@@ -36265,7 +36265,7 @@
         <v>10</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q20">
         <v>9</v>
@@ -36354,7 +36354,7 @@
         <v>10</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q21">
         <v>9</v>
@@ -36443,7 +36443,7 @@
         <v>6</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q22">
         <v>7</v>
@@ -36464,7 +36464,7 @@
         <v>7</v>
       </c>
       <c r="W22">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="X22">
         <v>6</v>
@@ -36532,7 +36532,7 @@
         <v>10</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q23">
         <v>9</v>
@@ -36553,7 +36553,7 @@
         <v>9</v>
       </c>
       <c r="W23">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="X23">
         <v>8</v>
@@ -36621,7 +36621,7 @@
         <v>7</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q24">
         <v>5</v>
@@ -36710,7 +36710,7 @@
         <v>9</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q25">
         <v>7</v>
@@ -36799,7 +36799,7 @@
         <v>7</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q26">
         <v>7</v>
@@ -36888,7 +36888,7 @@
         <v>6</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q27">
         <v>5</v>
@@ -37138,7 +37138,7 @@
         <v>7</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T4">
         <v>8</v>
@@ -37147,7 +37147,7 @@
         <v>7</v>
       </c>
       <c r="V4">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W4">
         <v>8</v>
@@ -37227,7 +37227,7 @@
         <v>7</v>
       </c>
       <c r="S5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T5">
         <v>8</v>
@@ -37236,7 +37236,7 @@
         <v>5</v>
       </c>
       <c r="V5">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W5">
         <v>7</v>
@@ -37248,7 +37248,7 @@
         <v>6</v>
       </c>
       <c r="Z5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA5">
         <v>6</v>
@@ -37316,7 +37316,7 @@
         <v>6</v>
       </c>
       <c r="S6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T6">
         <v>6</v>
@@ -37325,7 +37325,7 @@
         <v>10</v>
       </c>
       <c r="V6">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W6">
         <v>8</v>
@@ -37337,7 +37337,7 @@
         <v>5</v>
       </c>
       <c r="Z6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA6">
         <v>6</v>
@@ -37405,7 +37405,7 @@
         <v>6</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T7">
         <v>8</v>
@@ -37414,7 +37414,7 @@
         <v>8</v>
       </c>
       <c r="V7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W7">
         <v>6</v>
@@ -37426,7 +37426,7 @@
         <v>6</v>
       </c>
       <c r="Z7">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AA7">
         <v>6</v>
@@ -37494,7 +37494,7 @@
         <v>6</v>
       </c>
       <c r="S8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T8">
         <v>7</v>
@@ -37503,7 +37503,7 @@
         <v>10</v>
       </c>
       <c r="V8">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W8">
         <v>7</v>
@@ -37583,7 +37583,7 @@
         <v>8</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T9">
         <v>10</v>
@@ -37592,7 +37592,7 @@
         <v>9</v>
       </c>
       <c r="V9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W9">
         <v>9</v>
@@ -37604,7 +37604,7 @@
         <v>7</v>
       </c>
       <c r="Z9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA9">
         <v>8</v>
@@ -37613,7 +37613,7 @@
         <v>8</v>
       </c>
       <c r="AC9">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:29">
@@ -37672,7 +37672,7 @@
         <v>7</v>
       </c>
       <c r="S10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T10">
         <v>8</v>
@@ -37681,7 +37681,7 @@
         <v>7</v>
       </c>
       <c r="V10">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W10">
         <v>8</v>
@@ -37693,7 +37693,7 @@
         <v>6</v>
       </c>
       <c r="Z10">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA10">
         <v>7</v>
@@ -37761,7 +37761,7 @@
         <v>5</v>
       </c>
       <c r="S11">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T11">
         <v>10</v>
@@ -37770,7 +37770,7 @@
         <v>9</v>
       </c>
       <c r="V11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W11">
         <v>7</v>
@@ -37782,7 +37782,7 @@
         <v>5</v>
       </c>
       <c r="Z11">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AA11">
         <v>7</v>
@@ -37850,7 +37850,7 @@
         <v>6</v>
       </c>
       <c r="S12">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T12">
         <v>9</v>
@@ -37859,7 +37859,7 @@
         <v>7</v>
       </c>
       <c r="V12">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W12">
         <v>7</v>
@@ -37871,7 +37871,7 @@
         <v>6</v>
       </c>
       <c r="Z12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA12">
         <v>6</v>
@@ -37880,7 +37880,7 @@
         <v>9</v>
       </c>
       <c r="AC12">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:29">
@@ -37939,7 +37939,7 @@
         <v>7</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T13">
         <v>7</v>
@@ -37948,7 +37948,7 @@
         <v>8</v>
       </c>
       <c r="V13">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W13">
         <v>7</v>
@@ -37960,7 +37960,7 @@
         <v>6</v>
       </c>
       <c r="Z13">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA13">
         <v>8</v>
@@ -38028,7 +38028,7 @@
         <v>7</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T14">
         <v>10</v>
@@ -38037,7 +38037,7 @@
         <v>6</v>
       </c>
       <c r="V14">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W14">
         <v>9</v>
@@ -38117,7 +38117,7 @@
         <v>5</v>
       </c>
       <c r="S15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T15">
         <v>7</v>
@@ -38126,7 +38126,7 @@
         <v>8</v>
       </c>
       <c r="V15">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W15">
         <v>8</v>
@@ -38138,7 +38138,7 @@
         <v>5</v>
       </c>
       <c r="Z15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA15">
         <v>6</v>
@@ -38206,7 +38206,7 @@
         <v>7</v>
       </c>
       <c r="S16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T16">
         <v>9</v>
@@ -38215,7 +38215,7 @@
         <v>9</v>
       </c>
       <c r="V16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W16">
         <v>9</v>
@@ -38227,7 +38227,7 @@
         <v>7</v>
       </c>
       <c r="Z16">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA16">
         <v>9</v>
@@ -38295,7 +38295,7 @@
         <v>5</v>
       </c>
       <c r="S17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T17">
         <v>8</v>
@@ -38304,7 +38304,7 @@
         <v>8</v>
       </c>
       <c r="V17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W17">
         <v>7</v>
@@ -38384,7 +38384,7 @@
         <v>6</v>
       </c>
       <c r="S18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T18">
         <v>10</v>
@@ -38393,7 +38393,7 @@
         <v>8</v>
       </c>
       <c r="V18">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W18">
         <v>9</v>
@@ -38405,7 +38405,7 @@
         <v>6</v>
       </c>
       <c r="Z18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA18">
         <v>9</v>
@@ -38473,7 +38473,7 @@
         <v>8</v>
       </c>
       <c r="S19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T19">
         <v>8</v>
@@ -38482,7 +38482,7 @@
         <v>9</v>
       </c>
       <c r="V19">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W19">
         <v>8</v>
@@ -38494,7 +38494,7 @@
         <v>6</v>
       </c>
       <c r="Z19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AA19">
         <v>6</v>
@@ -38562,7 +38562,7 @@
         <v>5</v>
       </c>
       <c r="S20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T20">
         <v>8</v>
@@ -38571,7 +38571,7 @@
         <v>8</v>
       </c>
       <c r="V20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W20">
         <v>6</v>
@@ -38583,7 +38583,7 @@
         <v>5</v>
       </c>
       <c r="Z20">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA20">
         <v>7</v>
@@ -38592,7 +38592,7 @@
         <v>6</v>
       </c>
       <c r="AC20">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:29">
@@ -38651,7 +38651,7 @@
         <v>4</v>
       </c>
       <c r="S21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T21">
         <v>9</v>
@@ -38660,7 +38660,7 @@
         <v>7</v>
       </c>
       <c r="V21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W21">
         <v>8</v>
@@ -38672,7 +38672,7 @@
         <v>5</v>
       </c>
       <c r="Z21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA21">
         <v>7</v>
@@ -38681,7 +38681,7 @@
         <v>7</v>
       </c>
       <c r="AC21">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:29">
@@ -38740,7 +38740,7 @@
         <v>7</v>
       </c>
       <c r="S22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T22">
         <v>9</v>
@@ -38749,7 +38749,7 @@
         <v>10</v>
       </c>
       <c r="V22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="W22">
         <v>7</v>
@@ -38770,7 +38770,7 @@
         <v>7</v>
       </c>
       <c r="AC22">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:29">
@@ -38829,7 +38829,7 @@
         <v>6</v>
       </c>
       <c r="S23">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T23">
         <v>7</v>
@@ -38838,7 +38838,7 @@
         <v>7</v>
       </c>
       <c r="V23">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W23">
         <v>8</v>
@@ -38850,7 +38850,7 @@
         <v>6</v>
       </c>
       <c r="Z23">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AA23">
         <v>6</v>
@@ -38918,7 +38918,7 @@
         <v>0</v>
       </c>
       <c r="S24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T24">
         <v>5</v>
@@ -38927,7 +38927,7 @@
         <v>5</v>
       </c>
       <c r="V24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W24">
         <v>5</v>
@@ -39007,7 +39007,7 @@
         <v>7</v>
       </c>
       <c r="S25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T25">
         <v>7</v>
@@ -39016,7 +39016,7 @@
         <v>4</v>
       </c>
       <c r="V25">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W25">
         <v>8</v>
@@ -39028,7 +39028,7 @@
         <v>7</v>
       </c>
       <c r="Z25">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA25">
         <v>7</v>
@@ -39096,7 +39096,7 @@
         <v>6</v>
       </c>
       <c r="S26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T26">
         <v>9</v>
@@ -39105,7 +39105,7 @@
         <v>10</v>
       </c>
       <c r="V26">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W26">
         <v>9</v>
@@ -39117,7 +39117,7 @@
         <v>6</v>
       </c>
       <c r="Z26">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA26">
         <v>8</v>
@@ -39185,7 +39185,7 @@
         <v>4</v>
       </c>
       <c r="S27">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T27">
         <v>5</v>
@@ -39194,7 +39194,7 @@
         <v>5</v>
       </c>
       <c r="V27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W27">
         <v>7</v>
@@ -39206,7 +39206,7 @@
         <v>5</v>
       </c>
       <c r="Z27">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA27">
         <v>5</v>
@@ -39215,7 +39215,7 @@
         <v>5</v>
       </c>
       <c r="AC27">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:29">
@@ -39274,7 +39274,7 @@
         <v>4</v>
       </c>
       <c r="S28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T28">
         <v>5</v>
@@ -39283,7 +39283,7 @@
         <v>5</v>
       </c>
       <c r="V28">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W28">
         <v>5</v>
@@ -39363,7 +39363,7 @@
         <v>7</v>
       </c>
       <c r="S29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T29">
         <v>5</v>
@@ -39372,7 +39372,7 @@
         <v>5</v>
       </c>
       <c r="V29">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W29">
         <v>5</v>
@@ -39384,7 +39384,7 @@
         <v>5</v>
       </c>
       <c r="Z29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA29">
         <v>5</v>
@@ -39452,7 +39452,7 @@
         <v>9</v>
       </c>
       <c r="S30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T30">
         <v>8</v>
@@ -39461,7 +39461,7 @@
         <v>9</v>
       </c>
       <c r="V30">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W30">
         <v>8</v>
@@ -39473,7 +39473,7 @@
         <v>7</v>
       </c>
       <c r="Z30">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA30">
         <v>8</v>
@@ -39541,7 +39541,7 @@
         <v>0</v>
       </c>
       <c r="S31">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T31">
         <v>5</v>
@@ -39550,7 +39550,7 @@
         <v>7</v>
       </c>
       <c r="V31">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W31">
         <v>6</v>
@@ -39630,7 +39630,7 @@
         <v>7</v>
       </c>
       <c r="S32">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T32">
         <v>10</v>
@@ -39639,7 +39639,7 @@
         <v>6</v>
       </c>
       <c r="V32">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W32">
         <v>8</v>
@@ -39651,7 +39651,7 @@
         <v>6</v>
       </c>
       <c r="Z32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA32">
         <v>9</v>
@@ -39719,7 +39719,7 @@
         <v>10</v>
       </c>
       <c r="S33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T33">
         <v>10</v>
@@ -39728,7 +39728,7 @@
         <v>10</v>
       </c>
       <c r="V33">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W33">
         <v>10</v>
@@ -39808,7 +39808,7 @@
         <v>3</v>
       </c>
       <c r="S34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T34">
         <v>5</v>
@@ -39817,7 +39817,7 @@
         <v>5</v>
       </c>
       <c r="V34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W34">
         <v>5</v>
@@ -39829,7 +39829,7 @@
         <v>5</v>
       </c>
       <c r="Z34">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA34">
         <v>5</v>
@@ -39897,7 +39897,7 @@
         <v>7</v>
       </c>
       <c r="S35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T35">
         <v>10</v>
@@ -39906,7 +39906,7 @@
         <v>8</v>
       </c>
       <c r="V35">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W35">
         <v>8</v>
@@ -39986,7 +39986,7 @@
         <v>5</v>
       </c>
       <c r="S36">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T36">
         <v>8</v>
@@ -39995,7 +39995,7 @@
         <v>7</v>
       </c>
       <c r="V36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W36">
         <v>5</v>
@@ -40007,7 +40007,7 @@
         <v>5</v>
       </c>
       <c r="Z36">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA36">
         <v>6</v>
@@ -40075,7 +40075,7 @@
         <v>8</v>
       </c>
       <c r="S37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T37">
         <v>10</v>
@@ -40084,7 +40084,7 @@
         <v>10</v>
       </c>
       <c r="V37">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W37">
         <v>9</v>
@@ -40096,7 +40096,7 @@
         <v>6</v>
       </c>
       <c r="Z37">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA37">
         <v>10</v>
@@ -40164,7 +40164,7 @@
         <v>8</v>
       </c>
       <c r="S38">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T38">
         <v>8</v>
@@ -40173,7 +40173,7 @@
         <v>9</v>
       </c>
       <c r="V38">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="W38">
         <v>6</v>
@@ -40253,7 +40253,7 @@
         <v>6</v>
       </c>
       <c r="S39">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T39">
         <v>7</v>
@@ -40262,7 +40262,7 @@
         <v>9</v>
       </c>
       <c r="V39">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="W39">
         <v>7</v>
@@ -40274,7 +40274,7 @@
         <v>6</v>
       </c>
       <c r="Z39">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA39">
         <v>6</v>
@@ -40283,7 +40283,7 @@
         <v>7</v>
       </c>
       <c r="AC39">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:29">
@@ -40342,7 +40342,7 @@
         <v>5</v>
       </c>
       <c r="S40">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T40">
         <v>5</v>
@@ -40351,7 +40351,7 @@
         <v>6</v>
       </c>
       <c r="V40">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W40">
         <v>7</v>
@@ -40431,7 +40431,7 @@
         <v>8</v>
       </c>
       <c r="S41">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T41">
         <v>8</v>
@@ -40440,7 +40440,7 @@
         <v>5</v>
       </c>
       <c r="V41">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W41">
         <v>5</v>
@@ -40452,7 +40452,7 @@
         <v>5</v>
       </c>
       <c r="Z41">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA41">
         <v>6</v>
@@ -40520,7 +40520,7 @@
         <v>6</v>
       </c>
       <c r="S42">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T42">
         <v>7</v>
@@ -40529,7 +40529,7 @@
         <v>7</v>
       </c>
       <c r="V42">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="W42">
         <v>8</v>
@@ -40541,7 +40541,7 @@
         <v>6</v>
       </c>
       <c r="Z42">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA42">
         <v>6</v>
@@ -40761,7 +40761,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T4">
         <v>5</v>
@@ -40850,7 +40850,7 @@
         <v>9</v>
       </c>
       <c r="S5">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T5">
         <v>8</v>
@@ -40871,7 +40871,7 @@
         <v>7</v>
       </c>
       <c r="Z5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA5">
         <v>8</v>
@@ -40930,7 +40930,7 @@
         <v>5</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q6">
         <v>8</v>
@@ -40939,7 +40939,7 @@
         <v>8</v>
       </c>
       <c r="S6">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T6">
         <v>5</v>
@@ -40951,7 +40951,7 @@
         <v>5</v>
       </c>
       <c r="W6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="X6">
         <v>8</v>
@@ -41028,7 +41028,7 @@
         <v>8</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T7">
         <v>9</v>
@@ -41049,7 +41049,7 @@
         <v>7</v>
       </c>
       <c r="Z7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA7">
         <v>8</v>
@@ -41117,7 +41117,7 @@
         <v>7</v>
       </c>
       <c r="S8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T8">
         <v>8</v>
@@ -41206,7 +41206,7 @@
         <v>9</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T9">
         <v>9</v>
@@ -41295,7 +41295,7 @@
         <v>8</v>
       </c>
       <c r="S10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T10">
         <v>8</v>
@@ -41316,7 +41316,7 @@
         <v>7</v>
       </c>
       <c r="Z10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA10">
         <v>6</v>
@@ -41375,7 +41375,7 @@
         <v>6</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q11">
         <v>5</v>
@@ -41384,7 +41384,7 @@
         <v>6</v>
       </c>
       <c r="S11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T11">
         <v>5</v>
@@ -41405,7 +41405,7 @@
         <v>7</v>
       </c>
       <c r="Z11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA11">
         <v>6</v>
@@ -41473,7 +41473,7 @@
         <v>7</v>
       </c>
       <c r="S12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T12">
         <v>6</v>
@@ -41494,7 +41494,7 @@
         <v>7</v>
       </c>
       <c r="Z12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA12">
         <v>7</v>
@@ -41562,7 +41562,7 @@
         <v>4</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T13">
         <v>10</v>
@@ -41583,7 +41583,7 @@
         <v>5</v>
       </c>
       <c r="Z13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA13">
         <v>8</v>
@@ -41651,7 +41651,7 @@
         <v>5</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T14">
         <v>8</v>
@@ -41740,7 +41740,7 @@
         <v>6</v>
       </c>
       <c r="S15">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T15">
         <v>7</v>
@@ -41829,7 +41829,7 @@
         <v>4</v>
       </c>
       <c r="S16">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="T16">
         <v>6</v>
@@ -41918,7 +41918,7 @@
         <v>10</v>
       </c>
       <c r="S17">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T17">
         <v>9</v>
@@ -42007,7 +42007,7 @@
         <v>6</v>
       </c>
       <c r="S18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T18">
         <v>8</v>
@@ -42028,7 +42028,7 @@
         <v>6</v>
       </c>
       <c r="Z18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA18">
         <v>6</v>
@@ -42096,7 +42096,7 @@
         <v>7</v>
       </c>
       <c r="S19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T19">
         <v>7</v>
@@ -42117,7 +42117,7 @@
         <v>6</v>
       </c>
       <c r="Z19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA19">
         <v>6</v>
@@ -42185,7 +42185,7 @@
         <v>0</v>
       </c>
       <c r="S20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T20">
         <v>5</v>
@@ -42274,7 +42274,7 @@
         <v>7</v>
       </c>
       <c r="S21">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T21">
         <v>8</v>
@@ -42295,7 +42295,7 @@
         <v>6</v>
       </c>
       <c r="Z21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA21">
         <v>7</v>
@@ -42363,7 +42363,7 @@
         <v>4</v>
       </c>
       <c r="S22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T22">
         <v>5</v>
@@ -42384,7 +42384,7 @@
         <v>5</v>
       </c>
       <c r="Z22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA22">
         <v>5</v>
@@ -42443,7 +42443,7 @@
         <v>5</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>6</v>
       </c>
       <c r="Q23">
         <v>8</v>
@@ -42452,7 +42452,7 @@
         <v>7</v>
       </c>
       <c r="S23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T23">
         <v>8</v>
@@ -42473,7 +42473,7 @@
         <v>6</v>
       </c>
       <c r="Z23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA23">
         <v>7</v>
@@ -42541,7 +42541,7 @@
         <v>5</v>
       </c>
       <c r="S24">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T24">
         <v>8</v>
@@ -42562,7 +42562,7 @@
         <v>5</v>
       </c>
       <c r="Z24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA24">
         <v>6</v>
@@ -42630,7 +42630,7 @@
         <v>6</v>
       </c>
       <c r="S25">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T25">
         <v>8</v>
@@ -42651,7 +42651,7 @@
         <v>7</v>
       </c>
       <c r="Z25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA25">
         <v>8</v>
@@ -42719,7 +42719,7 @@
         <v>6</v>
       </c>
       <c r="S26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T26">
         <v>8</v>
@@ -42740,7 +42740,7 @@
         <v>6</v>
       </c>
       <c r="Z26">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA26">
         <v>6</v>
@@ -42808,7 +42808,7 @@
         <v>4</v>
       </c>
       <c r="S27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T27">
         <v>8</v>
@@ -42829,7 +42829,7 @@
         <v>5</v>
       </c>
       <c r="Z27">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA27">
         <v>7</v>
@@ -42897,7 +42897,7 @@
         <v>4</v>
       </c>
       <c r="S28">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T28">
         <v>9</v>
@@ -42918,7 +42918,7 @@
         <v>5</v>
       </c>
       <c r="Z28">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA28">
         <v>9</v>
@@ -42986,7 +42986,7 @@
         <v>5</v>
       </c>
       <c r="S29">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T29">
         <v>7</v>
@@ -43007,7 +43007,7 @@
         <v>5</v>
       </c>
       <c r="Z29">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA29">
         <v>7</v>
@@ -43075,7 +43075,7 @@
         <v>7</v>
       </c>
       <c r="S30">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T30">
         <v>10</v>
@@ -43096,7 +43096,7 @@
         <v>7</v>
       </c>
       <c r="Z30">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA30">
         <v>9</v>
@@ -43164,7 +43164,7 @@
         <v>7</v>
       </c>
       <c r="S31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T31">
         <v>9</v>
@@ -43253,7 +43253,7 @@
         <v>0</v>
       </c>
       <c r="S32">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T32">
         <v>5</v>
@@ -43342,7 +43342,7 @@
         <v>8</v>
       </c>
       <c r="S33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T33">
         <v>10</v>
@@ -43431,7 +43431,7 @@
         <v>6</v>
       </c>
       <c r="S34">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T34">
         <v>6</v>
@@ -43520,7 +43520,7 @@
         <v>10</v>
       </c>
       <c r="S35">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T35">
         <v>8</v>
@@ -43541,7 +43541,7 @@
         <v>5</v>
       </c>
       <c r="Z35">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA35">
         <v>8</v>
@@ -43600,7 +43600,7 @@
         <v>5</v>
       </c>
       <c r="P36">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="Q36">
         <v>5</v>
@@ -43609,7 +43609,7 @@
         <v>5</v>
       </c>
       <c r="S36">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T36">
         <v>5</v>
@@ -43698,7 +43698,7 @@
         <v>7</v>
       </c>
       <c r="S37">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T37">
         <v>8</v>
@@ -43719,7 +43719,7 @@
         <v>6</v>
       </c>
       <c r="Z37">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA37">
         <v>6</v>
@@ -43787,7 +43787,7 @@
         <v>7</v>
       </c>
       <c r="S38">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T38">
         <v>5</v>
@@ -43876,7 +43876,7 @@
         <v>9</v>
       </c>
       <c r="S39">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T39">
         <v>8</v>
@@ -43897,7 +43897,7 @@
         <v>7</v>
       </c>
       <c r="Z39">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA39">
         <v>7</v>
@@ -43965,7 +43965,7 @@
         <v>4</v>
       </c>
       <c r="S40">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T40">
         <v>8</v>
@@ -43986,7 +43986,7 @@
         <v>5</v>
       </c>
       <c r="Z40">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA40">
         <v>6</v>
@@ -44054,7 +44054,7 @@
         <v>10</v>
       </c>
       <c r="S41">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T41">
         <v>8</v>
@@ -44075,7 +44075,7 @@
         <v>8</v>
       </c>
       <c r="Z41">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA41">
         <v>7</v>
@@ -44143,7 +44143,7 @@
         <v>0</v>
       </c>
       <c r="S42">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T42">
         <v>5</v>
@@ -44384,7 +44384,7 @@
         <v>9</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T4">
         <v>8</v>
@@ -44405,7 +44405,7 @@
         <v>8</v>
       </c>
       <c r="Z4">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA4">
         <v>9</v>
@@ -44473,7 +44473,7 @@
         <v>7</v>
       </c>
       <c r="S5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T5">
         <v>7</v>
@@ -44494,7 +44494,7 @@
         <v>6</v>
       </c>
       <c r="Z5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA5">
         <v>7</v>
@@ -44562,7 +44562,7 @@
         <v>7</v>
       </c>
       <c r="S6">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T6">
         <v>7</v>
@@ -44583,7 +44583,7 @@
         <v>7</v>
       </c>
       <c r="Z6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA6">
         <v>6</v>
@@ -44651,7 +44651,7 @@
         <v>4</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T7">
         <v>5</v>
@@ -44672,7 +44672,7 @@
         <v>5</v>
       </c>
       <c r="Z7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA7">
         <v>5</v>
@@ -44740,7 +44740,7 @@
         <v>7</v>
       </c>
       <c r="S8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T8">
         <v>7</v>
@@ -44761,7 +44761,7 @@
         <v>6</v>
       </c>
       <c r="Z8">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AA8">
         <v>7</v>
@@ -44829,7 +44829,7 @@
         <v>7</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T9">
         <v>5</v>
@@ -44918,7 +44918,7 @@
         <v>4</v>
       </c>
       <c r="S10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T10">
         <v>5</v>
@@ -44939,7 +44939,7 @@
         <v>5</v>
       </c>
       <c r="Z10">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA10">
         <v>5</v>
@@ -45007,7 +45007,7 @@
         <v>4</v>
       </c>
       <c r="S11">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T11">
         <v>5</v>
@@ -45096,7 +45096,7 @@
         <v>6</v>
       </c>
       <c r="S12">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T12">
         <v>7</v>
@@ -45117,7 +45117,7 @@
         <v>6</v>
       </c>
       <c r="Z12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA12">
         <v>6</v>
@@ -45185,7 +45185,7 @@
         <v>7</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T13">
         <v>8</v>
@@ -45274,7 +45274,7 @@
         <v>4</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T14">
         <v>5</v>
@@ -45295,7 +45295,7 @@
         <v>5</v>
       </c>
       <c r="Z14">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA14">
         <v>5</v>
@@ -45363,7 +45363,7 @@
         <v>4</v>
       </c>
       <c r="S15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T15">
         <v>5</v>
@@ -45384,7 +45384,7 @@
         <v>5</v>
       </c>
       <c r="Z15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA15">
         <v>5</v>
@@ -45452,7 +45452,7 @@
         <v>5</v>
       </c>
       <c r="S16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T16">
         <v>5</v>
@@ -45473,7 +45473,7 @@
         <v>5</v>
       </c>
       <c r="Z16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA16">
         <v>5</v>
@@ -45541,7 +45541,7 @@
         <v>4</v>
       </c>
       <c r="S17">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T17">
         <v>5</v>
@@ -45630,7 +45630,7 @@
         <v>8</v>
       </c>
       <c r="S18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T18">
         <v>7</v>
@@ -45651,7 +45651,7 @@
         <v>7</v>
       </c>
       <c r="Z18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA18">
         <v>6</v>
@@ -45719,7 +45719,7 @@
         <v>7</v>
       </c>
       <c r="S19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T19">
         <v>9</v>
@@ -45740,7 +45740,7 @@
         <v>7</v>
       </c>
       <c r="Z19">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AA19">
         <v>8</v>
@@ -45808,7 +45808,7 @@
         <v>5</v>
       </c>
       <c r="S20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T20">
         <v>5</v>
@@ -45897,7 +45897,7 @@
         <v>5</v>
       </c>
       <c r="S21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T21">
         <v>6</v>
@@ -45918,7 +45918,7 @@
         <v>6</v>
       </c>
       <c r="Z21">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA21">
         <v>7</v>
@@ -45986,7 +45986,7 @@
         <v>10</v>
       </c>
       <c r="S22">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T22">
         <v>10</v>
@@ -46075,7 +46075,7 @@
         <v>8</v>
       </c>
       <c r="S23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T23">
         <v>9</v>
@@ -46096,7 +46096,7 @@
         <v>7</v>
       </c>
       <c r="Z23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA23">
         <v>8</v>
@@ -46164,7 +46164,7 @@
         <v>0</v>
       </c>
       <c r="S24">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T24">
         <v>5</v>
@@ -46253,7 +46253,7 @@
         <v>0</v>
       </c>
       <c r="S25">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T25">
         <v>5</v>
@@ -46342,7 +46342,7 @@
         <v>6</v>
       </c>
       <c r="S26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T26">
         <v>7</v>
@@ -46431,7 +46431,7 @@
         <v>0</v>
       </c>
       <c r="S27">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T27">
         <v>5</v>
@@ -46520,7 +46520,7 @@
         <v>6</v>
       </c>
       <c r="S28">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T28">
         <v>5</v>
@@ -46541,7 +46541,7 @@
         <v>6</v>
       </c>
       <c r="Z28">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA28">
         <v>5</v>
@@ -46609,7 +46609,7 @@
         <v>4</v>
       </c>
       <c r="S29">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T29">
         <v>8</v>
@@ -46630,7 +46630,7 @@
         <v>5</v>
       </c>
       <c r="Z29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA29">
         <v>6</v>
@@ -46698,7 +46698,7 @@
         <v>7</v>
       </c>
       <c r="S30">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T30">
         <v>5</v>
@@ -46719,7 +46719,7 @@
         <v>6</v>
       </c>
       <c r="Z30">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA30">
         <v>5</v>
@@ -46787,7 +46787,7 @@
         <v>7</v>
       </c>
       <c r="S31">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T31">
         <v>6</v>
@@ -46808,7 +46808,7 @@
         <v>6</v>
       </c>
       <c r="Z31">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA31">
         <v>7</v>
@@ -46876,7 +46876,7 @@
         <v>4</v>
       </c>
       <c r="S32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T32">
         <v>6</v>
@@ -46965,7 +46965,7 @@
         <v>6</v>
       </c>
       <c r="S33">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T33">
         <v>8</v>
@@ -46986,7 +46986,7 @@
         <v>6</v>
       </c>
       <c r="Z33">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA33">
         <v>8</v>
@@ -47054,7 +47054,7 @@
         <v>9</v>
       </c>
       <c r="S34">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T34">
         <v>8</v>
@@ -47075,7 +47075,7 @@
         <v>7</v>
       </c>
       <c r="Z34">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA34">
         <v>7</v>
@@ -47143,7 +47143,7 @@
         <v>0</v>
       </c>
       <c r="S35">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T35">
         <v>5</v>
@@ -47232,7 +47232,7 @@
         <v>4</v>
       </c>
       <c r="S36">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T36">
         <v>6</v>
@@ -47253,7 +47253,7 @@
         <v>5</v>
       </c>
       <c r="Z36">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA36">
         <v>6</v>
@@ -47321,7 +47321,7 @@
         <v>4</v>
       </c>
       <c r="S37">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T37">
         <v>5</v>
@@ -47342,7 +47342,7 @@
         <v>5</v>
       </c>
       <c r="Z37">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA37">
         <v>5</v>
@@ -47410,7 +47410,7 @@
         <v>4</v>
       </c>
       <c r="S38">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T38">
         <v>5</v>
@@ -47431,7 +47431,7 @@
         <v>5</v>
       </c>
       <c r="Z38">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA38">
         <v>5</v>
@@ -47499,7 +47499,7 @@
         <v>5</v>
       </c>
       <c r="S39">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T39">
         <v>5</v>
@@ -47520,7 +47520,7 @@
         <v>5</v>
       </c>
       <c r="Z39">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA39">
         <v>5</v>
@@ -47588,7 +47588,7 @@
         <v>7</v>
       </c>
       <c r="S40">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T40">
         <v>5</v>
@@ -47609,7 +47609,7 @@
         <v>7</v>
       </c>
       <c r="Z40">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AA40">
         <v>5</v>
@@ -47829,7 +47829,7 @@
         <v>6</v>
       </c>
       <c r="S4">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T4">
         <v>8</v>
@@ -47850,7 +47850,7 @@
         <v>5</v>
       </c>
       <c r="Z4">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA4">
         <v>7</v>
@@ -47918,7 +47918,7 @@
         <v>7</v>
       </c>
       <c r="S5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T5">
         <v>7</v>
@@ -48007,7 +48007,7 @@
         <v>8</v>
       </c>
       <c r="S6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T6">
         <v>10</v>
@@ -48096,7 +48096,7 @@
         <v>9</v>
       </c>
       <c r="S7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T7">
         <v>10</v>
@@ -48185,7 +48185,7 @@
         <v>5</v>
       </c>
       <c r="S8">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T8">
         <v>5</v>
@@ -48206,7 +48206,7 @@
         <v>5</v>
       </c>
       <c r="Z8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA8">
         <v>5</v>
@@ -48274,7 +48274,7 @@
         <v>8</v>
       </c>
       <c r="S9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T9">
         <v>8</v>
@@ -48363,7 +48363,7 @@
         <v>10</v>
       </c>
       <c r="S10">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T10">
         <v>10</v>
@@ -48452,7 +48452,7 @@
         <v>0</v>
       </c>
       <c r="S11">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T11">
         <v>5</v>
@@ -48541,7 +48541,7 @@
         <v>7</v>
       </c>
       <c r="S12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T12">
         <v>6</v>
@@ -48562,7 +48562,7 @@
         <v>6</v>
       </c>
       <c r="Z12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA12">
         <v>6</v>
@@ -48630,7 +48630,7 @@
         <v>7</v>
       </c>
       <c r="S13">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T13">
         <v>8</v>
@@ -48651,7 +48651,7 @@
         <v>6</v>
       </c>
       <c r="Z13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA13">
         <v>6</v>
@@ -48719,7 +48719,7 @@
         <v>10</v>
       </c>
       <c r="S14">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T14">
         <v>9</v>
@@ -48740,7 +48740,7 @@
         <v>7</v>
       </c>
       <c r="Z14">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AA14">
         <v>7</v>
@@ -48808,7 +48808,7 @@
         <v>8</v>
       </c>
       <c r="S15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T15">
         <v>9</v>
@@ -48897,7 +48897,7 @@
         <v>8</v>
       </c>
       <c r="S16">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T16">
         <v>8</v>
@@ -48986,7 +48986,7 @@
         <v>10</v>
       </c>
       <c r="S17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="T17">
         <v>9</v>
@@ -49075,7 +49075,7 @@
         <v>6</v>
       </c>
       <c r="S18">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="T18">
         <v>7</v>
@@ -49096,7 +49096,7 @@
         <v>6</v>
       </c>
       <c r="Z18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA18">
         <v>6</v>
@@ -49164,7 +49164,7 @@
         <v>7</v>
       </c>
       <c r="S19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="T19">
         <v>8</v>
@@ -49185,7 +49185,7 @@
         <v>6</v>
       </c>
       <c r="Z19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA19">
         <v>6</v>
@@ -49253,7 +49253,7 @@
         <v>4</v>
       </c>
       <c r="S20">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T20">
         <v>5</v>
@@ -49342,7 +49342,7 @@
         <v>6</v>
       </c>
       <c r="S21">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="T21">
         <v>6</v>
@@ -49363,7 +49363,7 @@
         <v>6</v>
       </c>
       <c r="Z21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA21">
         <v>6</v>
@@ -49431,7 +49431,7 @@
         <v>5</v>
       </c>
       <c r="S22">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="T22">
         <v>5</v>
@@ -54695,7 +54695,7 @@
         <v>6</v>
       </c>
       <c r="R4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S4">
         <v>7</v>
@@ -54713,7 +54713,7 @@
         <v>6</v>
       </c>
       <c r="X4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Y4">
         <v>5</v>
@@ -54772,7 +54772,7 @@
         <v>8</v>
       </c>
       <c r="R5">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S5">
         <v>7</v>
@@ -54790,7 +54790,7 @@
         <v>8</v>
       </c>
       <c r="X5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y5">
         <v>7</v>
@@ -54849,7 +54849,7 @@
         <v>10</v>
       </c>
       <c r="R6">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S6">
         <v>9</v>
@@ -54867,7 +54867,7 @@
         <v>9</v>
       </c>
       <c r="X6">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y6">
         <v>7</v>
@@ -54926,7 +54926,7 @@
         <v>8</v>
       </c>
       <c r="R7">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S7">
         <v>7</v>
@@ -54944,7 +54944,7 @@
         <v>7</v>
       </c>
       <c r="X7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y7">
         <v>6</v>
@@ -55003,7 +55003,7 @@
         <v>10</v>
       </c>
       <c r="R8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S8">
         <v>10</v>
@@ -55021,7 +55021,7 @@
         <v>10</v>
       </c>
       <c r="X8">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y8">
         <v>9</v>
@@ -55080,7 +55080,7 @@
         <v>9</v>
       </c>
       <c r="R9">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S9">
         <v>6</v>
@@ -55157,7 +55157,7 @@
         <v>5</v>
       </c>
       <c r="R10">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S10">
         <v>3</v>
@@ -55234,7 +55234,7 @@
         <v>9</v>
       </c>
       <c r="R11">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S11">
         <v>6</v>
@@ -55311,7 +55311,7 @@
         <v>7</v>
       </c>
       <c r="R12">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S12">
         <v>3</v>
@@ -55329,7 +55329,7 @@
         <v>6</v>
       </c>
       <c r="X12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y12">
         <v>5</v>
@@ -55388,7 +55388,7 @@
         <v>10</v>
       </c>
       <c r="R13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S13">
         <v>10</v>
@@ -55465,7 +55465,7 @@
         <v>10</v>
       </c>
       <c r="R14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S14">
         <v>9</v>
@@ -55542,7 +55542,7 @@
         <v>8</v>
       </c>
       <c r="R15">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="S15">
         <v>5</v>
@@ -55619,7 +55619,7 @@
         <v>7</v>
       </c>
       <c r="R16">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S16">
         <v>9</v>
@@ -55637,7 +55637,7 @@
         <v>8</v>
       </c>
       <c r="X16">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y16">
         <v>8</v>
@@ -55696,7 +55696,7 @@
         <v>10</v>
       </c>
       <c r="R17">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S17">
         <v>8</v>
@@ -55714,7 +55714,7 @@
         <v>8</v>
       </c>
       <c r="X17">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y17">
         <v>8</v>
@@ -55773,7 +55773,7 @@
         <v>5</v>
       </c>
       <c r="R18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S18">
         <v>5</v>
@@ -55791,7 +55791,7 @@
         <v>5</v>
       </c>
       <c r="X18">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y18">
         <v>5</v>
@@ -55850,7 +55850,7 @@
         <v>10</v>
       </c>
       <c r="R19">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S19">
         <v>10</v>
@@ -55868,7 +55868,7 @@
         <v>8</v>
       </c>
       <c r="X19">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Y19">
         <v>9</v>
@@ -55927,7 +55927,7 @@
         <v>10</v>
       </c>
       <c r="R20">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S20">
         <v>6</v>
@@ -55945,7 +55945,7 @@
         <v>9</v>
       </c>
       <c r="X20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y20">
         <v>7</v>
@@ -56004,7 +56004,7 @@
         <v>8</v>
       </c>
       <c r="R21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S21">
         <v>7</v>
@@ -56022,7 +56022,7 @@
         <v>8</v>
       </c>
       <c r="X21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y21">
         <v>7</v>
@@ -56081,7 +56081,7 @@
         <v>5</v>
       </c>
       <c r="R22">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S22">
         <v>5</v>
@@ -56099,7 +56099,7 @@
         <v>5</v>
       </c>
       <c r="X22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y22">
         <v>5</v>
@@ -56158,7 +56158,7 @@
         <v>8</v>
       </c>
       <c r="R23">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S23">
         <v>7</v>
@@ -56176,7 +56176,7 @@
         <v>7</v>
       </c>
       <c r="X23">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Y23">
         <v>6</v>
@@ -56235,7 +56235,7 @@
         <v>8</v>
       </c>
       <c r="R24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S24">
         <v>9</v>
@@ -56312,7 +56312,7 @@
         <v>9</v>
       </c>
       <c r="R25">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="S25">
         <v>5</v>
@@ -56389,7 +56389,7 @@
         <v>6</v>
       </c>
       <c r="R26">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="S26">
         <v>7</v>
@@ -56407,7 +56407,7 @@
         <v>8</v>
       </c>
       <c r="X26">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Y26">
         <v>7</v>
@@ -56495,7 +56495,7 @@
         <v>10</v>
       </c>
       <c r="R28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="S28">
         <v>10</v>
@@ -58857,7 +58857,7 @@
         <v>9</v>
       </c>
       <c r="P4">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q4">
         <v>10</v>
@@ -58934,7 +58934,7 @@
         <v>5</v>
       </c>
       <c r="P5">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q5">
         <v>8</v>
@@ -58952,7 +58952,7 @@
         <v>7</v>
       </c>
       <c r="V5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="W5">
         <v>6</v>
@@ -59011,7 +59011,7 @@
         <v>10</v>
       </c>
       <c r="P6">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q6">
         <v>9</v>
@@ -59088,7 +59088,7 @@
         <v>8</v>
       </c>
       <c r="P7">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q7">
         <v>10</v>
@@ -59165,7 +59165,7 @@
         <v>8</v>
       </c>
       <c r="P8">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q8">
         <v>8</v>
@@ -59242,7 +59242,7 @@
         <v>9</v>
       </c>
       <c r="P9">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q9">
         <v>9</v>
@@ -59319,7 +59319,7 @@
         <v>7</v>
       </c>
       <c r="P10">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q10">
         <v>10</v>
@@ -59396,7 +59396,7 @@
         <v>8</v>
       </c>
       <c r="P11">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q11">
         <v>9</v>
@@ -59473,7 +59473,7 @@
         <v>6</v>
       </c>
       <c r="P12">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q12">
         <v>8</v>
@@ -59491,7 +59491,7 @@
         <v>8</v>
       </c>
       <c r="V12">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W12">
         <v>8</v>
@@ -59550,7 +59550,7 @@
         <v>10</v>
       </c>
       <c r="P13">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q13">
         <v>9</v>
@@ -59627,7 +59627,7 @@
         <v>10</v>
       </c>
       <c r="P14">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q14">
         <v>10</v>
@@ -59704,7 +59704,7 @@
         <v>9</v>
       </c>
       <c r="P15">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q15">
         <v>10</v>
@@ -59781,7 +59781,7 @@
         <v>6</v>
       </c>
       <c r="P16">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q16">
         <v>7</v>
@@ -59858,7 +59858,7 @@
         <v>8</v>
       </c>
       <c r="P17">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q17">
         <v>8</v>
@@ -59935,7 +59935,7 @@
         <v>9</v>
       </c>
       <c r="P18">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q18">
         <v>9</v>
@@ -59953,7 +59953,7 @@
         <v>8</v>
       </c>
       <c r="V18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W18">
         <v>7</v>
@@ -60012,7 +60012,7 @@
         <v>8</v>
       </c>
       <c r="P19">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q19">
         <v>8</v>
@@ -60030,7 +60030,7 @@
         <v>7</v>
       </c>
       <c r="V19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="W19">
         <v>8</v>
@@ -60089,7 +60089,7 @@
         <v>9</v>
       </c>
       <c r="P20">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q20">
         <v>8</v>
@@ -60166,7 +60166,7 @@
         <v>9</v>
       </c>
       <c r="P21">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q21">
         <v>9</v>
@@ -60243,7 +60243,7 @@
         <v>8</v>
       </c>
       <c r="P22">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q22">
         <v>10</v>
@@ -60320,7 +60320,7 @@
         <v>9</v>
       </c>
       <c r="P23">
-        <v>-1</v>
+        <v>7</v>
       </c>
       <c r="Q23">
         <v>9</v>
@@ -60397,7 +60397,7 @@
         <v>10</v>
       </c>
       <c r="P24">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q24">
         <v>9</v>
@@ -60474,7 +60474,7 @@
         <v>8</v>
       </c>
       <c r="P25">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q25">
         <v>8</v>
@@ -60551,7 +60551,7 @@
         <v>9</v>
       </c>
       <c r="P26">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q26">
         <v>8</v>
@@ -60628,7 +60628,7 @@
         <v>8</v>
       </c>
       <c r="P27">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q27">
         <v>9</v>
@@ -60646,7 +60646,7 @@
         <v>7</v>
       </c>
       <c r="V27">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W27">
         <v>8</v>
@@ -60705,7 +60705,7 @@
         <v>10</v>
       </c>
       <c r="P28">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q28">
         <v>10</v>
@@ -60782,7 +60782,7 @@
         <v>8</v>
       </c>
       <c r="P29">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q29">
         <v>9</v>
@@ -60859,7 +60859,7 @@
         <v>9</v>
       </c>
       <c r="P30">
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="Q30">
         <v>8</v>
@@ -60936,7 +60936,7 @@
         <v>8</v>
       </c>
       <c r="P31">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q31">
         <v>7</v>
@@ -60954,7 +60954,7 @@
         <v>8</v>
       </c>
       <c r="V31">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W31">
         <v>7</v>
@@ -61013,7 +61013,7 @@
         <v>10</v>
       </c>
       <c r="P32">
-        <v>-1</v>
+        <v>8</v>
       </c>
       <c r="Q32">
         <v>8</v>
@@ -61031,7 +61031,7 @@
         <v>8</v>
       </c>
       <c r="V32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="W32">
         <v>6</v>
@@ -61090,7 +61090,7 @@
         <v>10</v>
       </c>
       <c r="P33">
-        <v>-1</v>
+        <v>9</v>
       </c>
       <c r="Q33">
         <v>9</v>
@@ -67276,7 +67276,7 @@
         <v>7</v>
       </c>
       <c r="O6">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="P6">
         <v>10</v>
@@ -67294,7 +67294,7 @@
         <v>8</v>
       </c>
       <c r="U6">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V6">
         <v>9</v>
@@ -67353,7 +67353,7 @@
         <v>6</v>
       </c>
       <c r="O7">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P7">
         <v>5</v>
@@ -67371,7 +67371,7 @@
         <v>7</v>
       </c>
       <c r="U7">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V7">
         <v>5</v>
@@ -67661,7 +67661,7 @@
         <v>7</v>
       </c>
       <c r="O11">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="P11">
         <v>5</v>
@@ -67679,7 +67679,7 @@
         <v>8</v>
       </c>
       <c r="U11">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V11">
         <v>7</v>
@@ -67892,7 +67892,7 @@
         <v>7</v>
       </c>
       <c r="O14">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="P14">
         <v>5</v>
@@ -67910,7 +67910,7 @@
         <v>7</v>
       </c>
       <c r="U14">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V14">
         <v>5</v>
@@ -68046,7 +68046,7 @@
         <v>7</v>
       </c>
       <c r="O16">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="P16">
         <v>8</v>
@@ -68064,7 +68064,7 @@
         <v>6</v>
       </c>
       <c r="U16">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V16">
         <v>6</v>
@@ -69355,7 +69355,7 @@
         <v>8</v>
       </c>
       <c r="O33">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="P33">
         <v>7</v>
@@ -69373,7 +69373,7 @@
         <v>7</v>
       </c>
       <c r="U33">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V33">
         <v>6</v>
@@ -69509,7 +69509,7 @@
         <v>6</v>
       </c>
       <c r="O35">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="P35">
         <v>7</v>
@@ -69527,7 +69527,7 @@
         <v>6</v>
       </c>
       <c r="U35">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="V35">
         <v>6</v>

</xml_diff>